<commit_message>
continue enterprise build scripts
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v02.xlsx
+++ b/Excel/10_SolidWaste_WIP_v02.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FEE79C2-D82C-4A79-8E7F-0759F6054B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E5D735-7B3F-4223-9154-4EF731663506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="60" windowWidth="37950" windowHeight="20355" firstSheet="1" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12645" firstSheet="1" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -231,6 +231,10 @@
     <definedName name="Step1">#REF!</definedName>
     <definedName name="Step2">#REF!</definedName>
     <definedName name="Step3">#REF!</definedName>
+    <definedName name="Table_E_g_offsite">'10.1.1-2 Solid waste treatment'!$D$156:$E$190</definedName>
+    <definedName name="Table_E_g_onsite">'10.1.1-2 Solid waste treatment'!$D$115:$E$149</definedName>
+    <definedName name="Table_V_w_t_offsite">'10.1.1-2 Solid waste treatment'!$D$58:$E$92</definedName>
+    <definedName name="Table_V_w_t_onsite">'10.1.1-2 Solid waste treatment'!$D$20:$E$54</definedName>
     <definedName name="VEERG_10_1_1_1__1_EmissionsFromWasteManagement_Scope1_Result_Method1">'10.1.1-2 Solid waste treatment'!$E$151</definedName>
     <definedName name="VEERG_10_1_1_1__1_EmissionsFromWasteManagement_Scope3_Result_Method1">'10.1.1-2 Solid waste treatment'!$E$192</definedName>
     <definedName name="WasteSolid_Equations.VEERG_10_1_1_1__1_EmissionsFromWasteManagement">_xlfn.LAMBDA(_xlpm.Q_wt,_xlpm.EF_wtg, _xlpm.Q_wt * _xlpm.EF_wtg)</definedName>
@@ -1777,7 +1781,7 @@
     </xf>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="31" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -1992,13 +1996,7 @@
     <xf numFmtId="0" fontId="45" fillId="4" borderId="2" xfId="64">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="56" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="8" applyFont="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2241,212 +2239,6 @@
           <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <family val="2"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -3323,6 +3115,212 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
@@ -4094,8 +4092,8 @@
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1790426" cy="312906"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="TextBox 5">
@@ -4302,7 +4300,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="TextBox 5">
@@ -4520,49 +4518,49 @@
     <tableColumn id="1" xr3:uid="{A2B430F3-D1CF-4DBE-B788-FF3C20E22F28}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3CDDB25-5D60-4029-A9DA-FCDF6DED306F}" name="MAT" totalsRowDxfId="61" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{C3CDDB25-5D60-4029-A9DA-FCDF6DED306F}" name="MAT" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9679764B-2260-453C-903D-6DDFD533890A}" name="MAP" totalsRowDxfId="60" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{9679764B-2260-453C-903D-6DDFD533890A}" name="MAP" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{E0B96EC6-4CC7-4E17-A726-BE318859D69B}" name="Frost days per year" totalsRowDxfId="59" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{E0B96EC6-4CC7-4E17-A726-BE318859D69B}" name="Frost days per year" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{99D9532F-D633-43D8-9E09-E4CDFE2DA99A}" name="Elevation" totalsRowDxfId="58" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{99D9532F-D633-43D8-9E09-E4CDFE2DA99A}" name="Elevation" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8EE4536F-60D5-4869-942F-180544702200}" name="MAP:PET" totalsRowDxfId="57" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{8EE4536F-60D5-4869-942F-180544702200}" name="MAP:PET" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{0FBAF10F-60EE-41D9-8B7E-87B685FD0BCF}" name="Min temp" totalsRowDxfId="56" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{0FBAF10F-60EE-41D9-8B7E-87B685FD0BCF}" name="Min temp" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{AAFC57CF-79ED-4BE2-8E90-4DD13CE49372}" name="Max temp" totalsRowDxfId="55" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{AAFC57CF-79ED-4BE2-8E90-4DD13CE49372}" name="Max temp" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{957B0523-D24F-4CDC-962F-4D2B1660898D}" name="Min rainfall" totalsRowDxfId="54" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{957B0523-D24F-4CDC-962F-4D2B1660898D}" name="Min rainfall" totalsRowDxfId="45" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{9E77BCDD-0E8C-4CF0-A1C5-85B308D8C052}" name="Max rainfall" totalsRowDxfId="53" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{9E77BCDD-0E8C-4CF0-A1C5-85B308D8C052}" name="Max rainfall" totalsRowDxfId="44" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{153CE395-CEED-4627-A2F5-BCEAC4C343B6}" name="Min frost days" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{153CE395-CEED-4627-A2F5-BCEAC4C343B6}" name="Min frost days" totalsRowDxfId="43" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{AF3247BE-0748-4077-A088-B88274EDB78C}" name="Max frost days" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{AF3247BE-0748-4077-A088-B88274EDB78C}" name="Max frost days" totalsRowDxfId="42" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{CA08E02B-2B67-4F32-A544-1CD765406C64}" name="Min elevation" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{CA08E02B-2B67-4F32-A544-1CD765406C64}" name="Min elevation" totalsRowDxfId="41" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{C508455B-0B90-439D-B21C-483306D70F51}" name="Max elevation" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{C508455B-0B90-439D-B21C-483306D70F51}" name="Max elevation" totalsRowDxfId="40" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{0F2F2640-788C-4191-ACF6-E8907F671213}" name="Min MAP:PET" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{0F2F2640-788C-4191-ACF6-E8907F671213}" name="Min MAP:PET" totalsRowDxfId="39" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{3886FF95-FFB6-4E58-8C4E-685D6C6DD1F1}" name="Max MAP:PET" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{3886FF95-FFB6-4E58-8C4E-685D6C6DD1F1}" name="Max MAP:PET" totalsRowDxfId="38" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4580,7 +4578,7 @@
     <tableColumn id="1" xr3:uid="{82668848-C846-4A8E-BEB5-6A099515513D}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F02B3268-15E1-4043-8BFA-C290D5EDE873}" name="Wet or Dry Zone" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{F02B3268-15E1-4043-8BFA-C290D5EDE873}" name="Wet or Dry Zone" totalsRowDxfId="37" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4686,7 +4684,7 @@
     <tableColumn id="1" xr3:uid="{A87C906C-828A-4DE3-9EB3-2FCA8EE8054D}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D7930F92-DBDF-4FD8-BF44-B4D67BB114A7}" name="FracWET" dataDxfId="45">
+    <tableColumn id="2" xr3:uid="{D7930F92-DBDF-4FD8-BF44-B4D67BB114A7}" name="FracWET" dataDxfId="36">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4736,13 +4734,13 @@
     <tableColumn id="1" xr3:uid="{27ECD0A0-9936-4A60-BCC5-02F0C62FDA6C}" name="Treatment type t">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B7AF1F5E-7BAC-4FF7-B59E-F905655514F2}" name="Waste type w" dataDxfId="21" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B7AF1F5E-7BAC-4FF7-B59E-F905655514F2}" name="Waste type w" dataDxfId="61" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{EEC6B364-DA50-41AA-A530-330FAEE98233}" name="EFwt" dataDxfId="20" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{EEC6B364-DA50-41AA-A530-330FAEE98233}" name="EFwt" dataDxfId="60" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{01FD94D2-85D3-4478-AB5E-04E4027C2978}" name="EF source" dataDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{01FD94D2-85D3-4478-AB5E-04E4027C2978}" name="EF source" dataDxfId="59" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4760,7 +4758,7 @@
     <tableColumn id="1" xr3:uid="{A399DD2C-2C8F-4921-AE90-4A605954450F}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{4E1AF06C-CDE4-4181-A993-5B0147FA6DF4}" name="FracWET" dataDxfId="44" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{4E1AF06C-CDE4-4181-A993-5B0147FA6DF4}" name="FracWET" dataDxfId="35" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4778,7 +4776,7 @@
     <tableColumn id="1" xr3:uid="{34C2D9DB-EED2-456F-BEA2-E59493B21593}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D0EDC8DD-395C-467A-B621-EFC3308C0D3A}" name="EFPRP" dataDxfId="43" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{D0EDC8DD-395C-467A-B621-EFC3308C0D3A}" name="EFPRP" dataDxfId="34" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4796,7 +4794,7 @@
     <tableColumn id="1" xr3:uid="{4295FB4A-FD24-4CF1-93B7-91D96C60BA18}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8C39FACA-411D-4F92-BE74-1F43448F529F}" name="Season" dataDxfId="42" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{8C39FACA-411D-4F92-BE74-1F43448F529F}" name="Season" dataDxfId="33" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4828,49 +4826,49 @@
     <tableColumn id="1" xr3:uid="{4888068E-C9B5-43FD-A916-9B7704914745}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B0FC6643-2FC3-4D44-9372-A36B5CC73DD7}" name="MAT (ºC)" dataDxfId="41" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B0FC6643-2FC3-4D44-9372-A36B5CC73DD7}" name="MAT (ºC)" dataDxfId="32" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0E51BB47-0324-4B13-8E89-7C9A5A09EC52}" name="Anaerobic lagoon" dataDxfId="40" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{0E51BB47-0324-4B13-8E89-7C9A5A09EC52}" name="Anaerobic lagoon" dataDxfId="31" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2312BF22-4881-442C-A8FD-F976FFCB79B7}" name="Digester / covered lagoons" dataDxfId="39" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{2312BF22-4881-442C-A8FD-F976FFCB79B7}" name="Digester / covered lagoons" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{1B70D6DD-C0F4-4284-8B69-FAEF867F1C6E}" name="Liquid systems" dataDxfId="38" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{1B70D6DD-C0F4-4284-8B69-FAEF867F1C6E}" name="Liquid systems" dataDxfId="29" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{2D0359C8-B312-4F0D-95CC-9F27DD9711CE}" name="Daily spread" dataDxfId="37" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{2D0359C8-B312-4F0D-95CC-9F27DD9711CE}" name="Daily spread" dataDxfId="28" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{5A63BD27-4E04-4451-82B2-4721FC78703D}" name="Composting (passive windrow)" dataDxfId="36" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{5A63BD27-4E04-4451-82B2-4721FC78703D}" name="Composting (passive windrow)" dataDxfId="27" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{9E6852C8-02EF-45CF-AE8F-A903AAB60C57}" name="Solid storage" dataDxfId="35" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{9E6852C8-02EF-45CF-AE8F-A903AAB60C57}" name="Solid storage" dataDxfId="26" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{74FF0616-5C4C-44A7-B4AB-CD29BC2285D1}" name="Pit storage" dataDxfId="34" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{74FF0616-5C4C-44A7-B4AB-CD29BC2285D1}" name="Pit storage" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{DC8F4831-78E1-4196-A054-44C26274DAB4}" name="Deep litter" dataDxfId="33" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{DC8F4831-78E1-4196-A054-44C26274DAB4}" name="Deep litter" dataDxfId="24" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{F4FFBAFB-4252-464A-913F-2B9A9D6C2256}" name="Poultry manure with bedding" dataDxfId="32" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{F4FFBAFB-4252-464A-913F-2B9A9D6C2256}" name="Poultry manure with bedding" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{9563BB03-86A6-4D44-AA7D-D448DA9F57D7}" name="Poultry manure without bedding" dataDxfId="31" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{9563BB03-86A6-4D44-AA7D-D448DA9F57D7}" name="Poultry manure without bedding" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{E7174980-0D39-4A0A-8B4A-73861E176A7D}" name="Direct processing" dataDxfId="30" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{E7174980-0D39-4A0A-8B4A-73861E176A7D}" name="Direct processing" dataDxfId="21" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{DD03C9E8-98A5-4484-920C-D6CF9FB7836F}" name="Direct application" dataDxfId="29" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{DD03C9E8-98A5-4484-920C-D6CF9FB7836F}" name="Direct application" dataDxfId="20" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{AFBD0566-0721-4CC3-A56B-684599A1581B}" name="Pasture range and paddock" dataDxfId="28" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{AFBD0566-0721-4CC3-A56B-684599A1581B}" name="Pasture range and paddock" dataDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{25C1DBBE-A111-4ED1-ABEE-B8DF2C7A1776}" name="MAT raw" dataDxfId="27" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{25C1DBBE-A111-4ED1-ABEE-B8DF2C7A1776}" name="MAT raw" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4888,7 +4886,7 @@
     <tableColumn id="1" xr3:uid="{E51F1B45-76B8-41BA-A4E8-39E28B5D22D8}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1C4AE05B-BAAC-4518-B0E9-FA3DAFBD52CD}" name="EFNi &amp; EFN2Oi" dataDxfId="26" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{1C4AE05B-BAAC-4518-B0E9-FA3DAFBD52CD}" name="EFNi &amp; EFN2Oi" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4906,7 +4904,7 @@
     <tableColumn id="1" xr3:uid="{E899A810-DA34-4DD3-9420-7017118A50BC}" name="Waste type w">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data(), Table_SourceData_WasteSolid_VolumeToMassConversion[[#Headers],[Waste type w]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EC8E9200-43B6-459C-B7A6-907C4A1A3CDE}" name="VTMw" dataDxfId="25" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{EC8E9200-43B6-459C-B7A6-907C4A1A3CDE}" name="VTMw" dataDxfId="58" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data(), Table_SourceData_WasteSolid_VolumeToMassConversion[[#Headers],[Waste type w]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4929,7 +4927,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}" name="Table_WasteTypes_Incineration" displayName="Table_WasteTypes_Incineration" ref="K16:K26" totalsRowShown="0" headerRowDxfId="24" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}" name="Table_WasteTypes_Incineration" displayName="Table_WasteTypes_Incineration" ref="K16:K26" totalsRowShown="0" headerRowDxfId="57" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="K16:K26" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
@@ -4943,12 +4941,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}" name="Table_WasteTypes_Composting" displayName="Table_WasteTypes_Composting" ref="M16:M21" totalsRowShown="0" headerRowDxfId="23" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}" name="Table_WasteTypes_Composting" displayName="Table_WasteTypes_Composting" ref="M16:M21" totalsRowShown="0" headerRowDxfId="56" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="M16:M21" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{5B9ABACD-52AE-4D64-BCA6-1DA86A1A3FC3}" name="Waste type w" totalsRowDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{5B9ABACD-52AE-4D64-BCA6-1DA86A1A3FC3}" name="Waste type w" totalsRowDxfId="55" dataCellStyle="Content normal">
       <calculatedColumnFormula>E40</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4957,12 +4955,12 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}" name="Table_WasteTypes_Anaerobicdigestion" displayName="Table_WasteTypes_Anaerobicdigestion" ref="O16:O21" totalsRowShown="0" headerRowDxfId="22" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}" name="Table_WasteTypes_Anaerobicdigestion" displayName="Table_WasteTypes_Anaerobicdigestion" ref="O16:O21" totalsRowShown="0" headerRowDxfId="54" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="O16:O21" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{2D7DB5DA-05BB-4621-B5A8-576415999BBC}" name="Waste type w" totalsRowDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{2D7DB5DA-05BB-4621-B5A8-576415999BBC}" name="Waste type w" totalsRowDxfId="53" dataCellStyle="Content normal">
       <calculatedColumnFormula>E46</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5595,7 +5593,7 @@
         <v>123</v>
       </c>
       <c r="E9" s="53">
-        <f>'10.1.1-2 Solid waste treatment'!E151</f>
+        <f>VEERG_10_1_1_1__1_EmissionsFromWasteManagement_Scope1_Result_Method1</f>
         <v>438.82805000000002</v>
       </c>
       <c r="F9" s="53">
@@ -5656,7 +5654,7 @@
         <v>123</v>
       </c>
       <c r="E13" s="53">
-        <f>'10.1.1-2 Solid waste treatment'!E192</f>
+        <f>VEERG_10_1_1_1__1_EmissionsFromWasteManagement_Scope3_Result_Method1</f>
         <v>441.15000000000003</v>
       </c>
       <c r="F13" s="53">
@@ -6726,7 +6724,7 @@
       <c r="G26" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="H26" s="77">
+      <c r="H26" s="75">
         <v>50</v>
       </c>
       <c r="I26" s="27" t="s">
@@ -6746,7 +6744,7 @@
       <c r="G27" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="H27" s="77">
+      <c r="H27" s="75">
         <v>50</v>
       </c>
       <c r="I27" s="27" t="s">
@@ -6766,7 +6764,7 @@
       <c r="G28" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="H28" s="77">
+      <c r="H28" s="75">
         <v>50</v>
       </c>
       <c r="I28" s="27" t="s">
@@ -6787,7 +6785,7 @@
       <c r="G29" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="H29" s="77">
+      <c r="H29" s="75">
         <v>50</v>
       </c>
       <c r="I29" s="27" t="s">
@@ -6809,7 +6807,7 @@
       <c r="G30" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="H30" s="77">
+      <c r="H30" s="75">
         <v>50</v>
       </c>
       <c r="I30" s="27" t="s">
@@ -6831,7 +6829,7 @@
       <c r="G31" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="H31" s="77">
+      <c r="H31" s="75">
         <v>50</v>
       </c>
       <c r="I31" s="27" t="s">
@@ -6853,7 +6851,7 @@
       <c r="G32" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="H32" s="77">
+      <c r="H32" s="75">
         <v>50</v>
       </c>
       <c r="I32" s="27" t="s">
@@ -9091,7 +9089,7 @@
         <v>50</v>
       </c>
       <c r="H116" s="28">
-        <f>I21</f>
+        <f t="shared" ref="H116:H135" si="0">I21</f>
         <v>25</v>
       </c>
       <c r="I116" s="28">
@@ -9120,11 +9118,11 @@
         <v>50</v>
       </c>
       <c r="H117" s="28">
-        <f>I22</f>
+        <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
       <c r="I117" s="28">
-        <f t="shared" ref="I117:I135" si="0">G117+H117</f>
+        <f t="shared" ref="I117:I135" si="1">G117+H117</f>
         <v>54.5</v>
       </c>
       <c r="J117" s="28" cm="1">
@@ -9149,11 +9147,11 @@
         <v>50</v>
       </c>
       <c r="H118" s="28">
-        <f>I23</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="I118" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>62</v>
       </c>
       <c r="J118" s="28" cm="1">
@@ -9178,11 +9176,11 @@
         <v>0</v>
       </c>
       <c r="H119" s="28">
-        <f>I24</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I119" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J119" s="28" cm="1">
@@ -9207,11 +9205,11 @@
         <v>0</v>
       </c>
       <c r="H120" s="28">
-        <f>I25</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I120" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J120" s="28" cm="1">
@@ -9236,11 +9234,11 @@
         <v>0</v>
       </c>
       <c r="H121" s="28">
-        <f>I26</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I121" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J121" s="28" cm="1">
@@ -9265,11 +9263,11 @@
         <v>0</v>
       </c>
       <c r="H122" s="28">
-        <f>I27</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I122" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J122" s="28" cm="1">
@@ -9294,11 +9292,11 @@
         <v>0</v>
       </c>
       <c r="H123" s="28">
-        <f>I28</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I123" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J123" s="28" cm="1">
@@ -9323,11 +9321,11 @@
         <v>0</v>
       </c>
       <c r="H124" s="28">
-        <f>I29</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I124" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J124" s="28" cm="1">
@@ -9352,11 +9350,11 @@
         <v>0</v>
       </c>
       <c r="H125" s="28">
-        <f>I30</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I125" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J125" s="28" cm="1">
@@ -9381,11 +9379,11 @@
         <v>0</v>
       </c>
       <c r="H126" s="28">
-        <f>I31</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I126" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J126" s="28" cm="1">
@@ -9409,7 +9407,7 @@
         <v>150</v>
       </c>
       <c r="H127" s="28" t="str">
-        <f>I32</f>
+        <f t="shared" si="0"/>
         <v>Not used</v>
       </c>
       <c r="I127" s="28">
@@ -9438,7 +9436,7 @@
         <v>0</v>
       </c>
       <c r="H128" s="28">
-        <f>I33</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I128" s="28" t="s">
@@ -9464,7 +9462,7 @@
         <v>50</v>
       </c>
       <c r="H129" s="28">
-        <f>I34</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="I129" s="28" t="s">
@@ -9490,7 +9488,7 @@
         <v>0</v>
       </c>
       <c r="H130" s="28">
-        <f>I35</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I130" s="28" t="s">
@@ -9516,7 +9514,7 @@
         <v>0</v>
       </c>
       <c r="H131" s="28">
-        <f>I36</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I131" s="28" t="s">
@@ -9542,11 +9540,11 @@
         <v>50</v>
       </c>
       <c r="H132" s="28">
-        <f>I37</f>
+        <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
       <c r="I132" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>54.5</v>
       </c>
       <c r="J132" s="28" cm="1">
@@ -9571,11 +9569,11 @@
         <v>0</v>
       </c>
       <c r="H133" s="28">
-        <f>I38</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I133" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J133" s="28" cm="1">
@@ -9600,11 +9598,11 @@
         <v>0</v>
       </c>
       <c r="H134" s="28">
-        <f>I39</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I134" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J134" s="28" cm="1">
@@ -9629,11 +9627,11 @@
         <v>0</v>
       </c>
       <c r="H135" s="28">
-        <f>I40</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I135" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J135" s="28" cm="1">
@@ -9662,11 +9660,11 @@
         <v>0</v>
       </c>
       <c r="H136" s="28">
-        <f t="shared" ref="G136:I149" si="1">I41</f>
+        <f t="shared" ref="H136:H149" si="2">I41</f>
         <v>0</v>
       </c>
       <c r="I136" s="28">
-        <f t="shared" ref="I136:I149" si="2">G136+H136</f>
+        <f t="shared" ref="I136:I137" si="3">G136+H136</f>
         <v>0</v>
       </c>
       <c r="J136" s="28" cm="1">
@@ -9691,11 +9689,11 @@
         <v>0</v>
       </c>
       <c r="H137" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I137" s="28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J137" s="28" cm="1">
@@ -9719,7 +9717,7 @@
         <v>150</v>
       </c>
       <c r="H138" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>Not used</v>
       </c>
       <c r="I138" s="28">
@@ -9748,7 +9746,7 @@
         <v>0</v>
       </c>
       <c r="H139" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="I139" s="28" t="s">
@@ -9774,7 +9772,7 @@
         <v>0</v>
       </c>
       <c r="H140" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I140" s="28" t="s">
@@ -9800,7 +9798,7 @@
         <v>0</v>
       </c>
       <c r="H141" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I141" s="28" t="s">
@@ -9826,7 +9824,7 @@
         <v>0</v>
       </c>
       <c r="H142" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I142" s="28" t="s">
@@ -9852,7 +9850,7 @@
         <v>0</v>
       </c>
       <c r="H143" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.5</v>
       </c>
       <c r="I143" s="28" t="s">
@@ -9877,7 +9875,7 @@
         <v>150</v>
       </c>
       <c r="H144" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>Not used</v>
       </c>
       <c r="I144" s="28">
@@ -9906,7 +9904,7 @@
         <v>0</v>
       </c>
       <c r="H145" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I145" s="28" t="s">
@@ -9932,7 +9930,7 @@
         <v>0</v>
       </c>
       <c r="H146" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I146" s="28" t="s">
@@ -9958,7 +9956,7 @@
         <v>0</v>
       </c>
       <c r="H147" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I147" s="28" t="s">
@@ -9984,7 +9982,7 @@
         <v>0</v>
       </c>
       <c r="H148" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I148" s="28" t="s">
@@ -10010,7 +10008,7 @@
         <v>0</v>
       </c>
       <c r="H149" s="28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I149" s="28" t="s">
@@ -10088,7 +10086,7 @@
         <v>50</v>
       </c>
       <c r="H157" s="28">
-        <f>I59</f>
+        <f t="shared" ref="H157:H176" si="4">I59</f>
         <v>25</v>
       </c>
       <c r="I157" s="28">
@@ -10117,11 +10115,11 @@
         <v>50</v>
       </c>
       <c r="H158" s="28">
-        <f>I60</f>
+        <f t="shared" si="4"/>
         <v>4.5</v>
       </c>
       <c r="I158" s="28">
-        <f t="shared" ref="I158:I176" si="3">G158+H158</f>
+        <f t="shared" ref="I158:I176" si="5">G158+H158</f>
         <v>54.5</v>
       </c>
       <c r="J158" s="28" cm="1">
@@ -10146,11 +10144,11 @@
         <v>50</v>
       </c>
       <c r="H159" s="28">
-        <f>I61</f>
+        <f t="shared" si="4"/>
         <v>12</v>
       </c>
       <c r="I159" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>62</v>
       </c>
       <c r="J159" s="28" cm="1">
@@ -10175,11 +10173,11 @@
         <v>0</v>
       </c>
       <c r="H160" s="28">
-        <f>I62</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I160" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J160" s="28" cm="1">
@@ -10204,11 +10202,11 @@
         <v>0</v>
       </c>
       <c r="H161" s="28">
-        <f>I63</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I161" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J161" s="28" cm="1">
@@ -10233,11 +10231,11 @@
         <v>0</v>
       </c>
       <c r="H162" s="28">
-        <f>I64</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I162" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J162" s="28" cm="1">
@@ -10262,11 +10260,11 @@
         <v>0</v>
       </c>
       <c r="H163" s="28">
-        <f>I65</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I163" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J163" s="28" cm="1">
@@ -10291,11 +10289,11 @@
         <v>0</v>
       </c>
       <c r="H164" s="28">
-        <f>I66</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I164" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J164" s="28" cm="1">
@@ -10320,11 +10318,11 @@
         <v>0</v>
       </c>
       <c r="H165" s="28">
-        <f>I67</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I165" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J165" s="28" cm="1">
@@ -10349,11 +10347,11 @@
         <v>0</v>
       </c>
       <c r="H166" s="28">
-        <f>I68</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I166" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J166" s="28" cm="1">
@@ -10378,11 +10376,11 @@
         <v>0</v>
       </c>
       <c r="H167" s="28">
-        <f>I69</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I167" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J167" s="28" cm="1">
@@ -10406,7 +10404,7 @@
         <v>150</v>
       </c>
       <c r="H168" s="28" t="str">
-        <f>I70</f>
+        <f t="shared" si="4"/>
         <v>Not used</v>
       </c>
       <c r="I168" s="28">
@@ -10435,7 +10433,7 @@
         <v>0</v>
       </c>
       <c r="H169" s="28">
-        <f>I71</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I169" s="28" t="s">
@@ -10461,7 +10459,7 @@
         <v>50</v>
       </c>
       <c r="H170" s="28">
-        <f>I72</f>
+        <f t="shared" si="4"/>
         <v>12</v>
       </c>
       <c r="I170" s="28" t="s">
@@ -10487,7 +10485,7 @@
         <v>0</v>
       </c>
       <c r="H171" s="28">
-        <f>I73</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I171" s="28" t="s">
@@ -10513,7 +10511,7 @@
         <v>0</v>
       </c>
       <c r="H172" s="28">
-        <f>I74</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I172" s="28" t="s">
@@ -10539,11 +10537,11 @@
         <v>0</v>
       </c>
       <c r="H173" s="28">
-        <f>I75</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I173" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J173" s="28" cm="1">
@@ -10568,11 +10566,11 @@
         <v>0</v>
       </c>
       <c r="H174" s="28">
-        <f>I76</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I174" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J174" s="28" cm="1">
@@ -10597,11 +10595,11 @@
         <v>0</v>
       </c>
       <c r="H175" s="28">
-        <f>I77</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I175" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J175" s="28" cm="1">
@@ -10626,11 +10624,11 @@
         <v>0</v>
       </c>
       <c r="H176" s="28">
-        <f>I78</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I176" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J176" s="28" cm="1">
@@ -10655,11 +10653,11 @@
         <v>0</v>
       </c>
       <c r="H177" s="28">
-        <f t="shared" ref="G177:H190" si="4">I79</f>
+        <f t="shared" ref="H177:H190" si="6">I79</f>
         <v>0</v>
       </c>
       <c r="I177" s="28">
-        <f t="shared" ref="I177:I190" si="5">G177+H177</f>
+        <f t="shared" ref="I177:I178" si="7">G177+H177</f>
         <v>0</v>
       </c>
       <c r="J177" s="28" cm="1">
@@ -10684,11 +10682,11 @@
         <v>0</v>
       </c>
       <c r="H178" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I178" s="28">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J178" s="28" cm="1">
@@ -10712,7 +10710,7 @@
         <v>150</v>
       </c>
       <c r="H179" s="28" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>Not used</v>
       </c>
       <c r="I179" s="28">
@@ -10741,7 +10739,7 @@
         <v>50</v>
       </c>
       <c r="H180" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I180" s="28" t="s">
@@ -10767,7 +10765,7 @@
         <v>0</v>
       </c>
       <c r="H181" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I181" s="28" t="s">
@@ -10793,7 +10791,7 @@
         <v>0</v>
       </c>
       <c r="H182" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I182" s="28" t="s">
@@ -10819,7 +10817,7 @@
         <v>0</v>
       </c>
       <c r="H183" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I183" s="28" t="s">
@@ -10845,7 +10843,7 @@
         <v>50</v>
       </c>
       <c r="H184" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I184" s="28" t="s">
@@ -10870,7 +10868,7 @@
         <v>150</v>
       </c>
       <c r="H185" s="28" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>Not used</v>
       </c>
       <c r="I185" s="28">
@@ -10899,7 +10897,7 @@
         <v>0</v>
       </c>
       <c r="H186" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I186" s="28" t="s">
@@ -10925,7 +10923,7 @@
         <v>0</v>
       </c>
       <c r="H187" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I187" s="28" t="s">
@@ -10951,7 +10949,7 @@
         <v>0</v>
       </c>
       <c r="H188" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I188" s="28" t="s">
@@ -10977,7 +10975,7 @@
         <v>0</v>
       </c>
       <c r="H189" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I189" s="28" t="s">
@@ -11003,7 +11001,7 @@
         <v>0</v>
       </c>
       <c r="H190" s="28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I190" s="28" t="s">
@@ -11354,7 +11352,7 @@
         <v>Food waste (including animal carcasses, spoiled animal feed or crop)</v>
       </c>
       <c r="K17" s="1" t="str">
-        <f>E29</f>
+        <f t="shared" ref="K17:K26" si="0">E29</f>
         <v>Food waste (including animal carcasses, spoiled animal feed or crop)</v>
       </c>
       <c r="M17" s="1" t="str">
@@ -11388,7 +11386,7 @@
         <v>Paper and cardboard</v>
       </c>
       <c r="K18" s="1" t="str">
-        <f>E30</f>
+        <f t="shared" si="0"/>
         <v>Green waste (including crop residues or prunings)</v>
       </c>
       <c r="M18" s="1" t="str">
@@ -11422,7 +11420,7 @@
         <v>Green waste (including crop residues or prunings)</v>
       </c>
       <c r="K19" s="1" t="str">
-        <f>E31</f>
+        <f t="shared" si="0"/>
         <v>Wood</v>
       </c>
       <c r="M19" s="1" t="str">
@@ -11457,7 +11455,7 @@
         <v>Wood</v>
       </c>
       <c r="K20" s="1" t="str">
-        <f>E32</f>
+        <f t="shared" si="0"/>
         <v>Sludge</v>
       </c>
       <c r="M20" s="1" t="str">
@@ -11492,7 +11490,7 @@
         <v>Textiles</v>
       </c>
       <c r="K21" s="1" t="str">
-        <f>E33</f>
+        <f t="shared" si="0"/>
         <v>Paper and cardboard</v>
       </c>
       <c r="M21" s="1" t="str">
@@ -11526,10 +11524,9 @@
         <v>Sludge</v>
       </c>
       <c r="K22" s="1" t="str">
-        <f>E34</f>
+        <f t="shared" si="0"/>
         <v>Textiles</v>
       </c>
-      <c r="M22" s="79"/>
     </row>
     <row r="23" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
@@ -11554,10 +11551,9 @@
         <v>Rubber and leather</v>
       </c>
       <c r="K23" s="1" t="str">
-        <f>E35</f>
+        <f t="shared" si="0"/>
         <v>Rubber and leather</v>
       </c>
-      <c r="M23" s="79"/>
     </row>
     <row r="24" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D24" s="1" t="str" cm="1">
@@ -11581,10 +11577,9 @@
         <v>Inert waste (including concrete, metal, plastic or glass)</v>
       </c>
       <c r="K24" s="1" t="str">
-        <f>E36</f>
+        <f t="shared" si="0"/>
         <v>Inert waste (including concrete, metal, plastic or glass)</v>
       </c>
-      <c r="M24" s="79"/>
     </row>
     <row r="25" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D25" s="1" t="str" cm="1">
@@ -11608,7 +11603,7 @@
         <v>Municipal solid waste</v>
       </c>
       <c r="K25" s="1" t="str">
-        <f>E37</f>
+        <f t="shared" si="0"/>
         <v>Municipal solid waste</v>
       </c>
     </row>
@@ -11634,7 +11629,7 @@
         <v>Commercial and industrial waste</v>
       </c>
       <c r="K26" s="1" t="str">
-        <f>E38</f>
+        <f t="shared" si="0"/>
         <v>Commercial and industrial waste</v>
       </c>
     </row>
@@ -11835,7 +11830,7 @@
         <f t="array" ref="F37">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>5.3699999999999998E-2</v>
       </c>
-      <c r="G37" s="78" t="str" cm="1">
+      <c r="G37" s="77" t="str" cm="1">
         <f t="array" ref="G37">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>NGAF 2025 Table 18</v>
       </c>
@@ -11853,7 +11848,7 @@
         <f t="array" ref="F38">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>1.649</v>
       </c>
-      <c r="G38" s="78" t="str" cm="1">
+      <c r="G38" s="77" t="str" cm="1">
         <f t="array" ref="G38">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>NGAF 2025 Table 18</v>
       </c>
@@ -11871,7 +11866,7 @@
         <f t="array" ref="F39">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>4.5999999999999999E-2</v>
       </c>
-      <c r="G39" s="78" t="str" cm="1">
+      <c r="G39" s="77" t="str" cm="1">
         <f t="array" ref="G39">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>NGAF 2025 Table 19</v>
       </c>
@@ -11889,7 +11884,7 @@
         <f t="array" ref="F40">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G40" s="78" t="str" cm="1">
+      <c r="G40" s="77" t="str" cm="1">
         <f t="array" ref="G40">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -11907,7 +11902,7 @@
         <f t="array" ref="F41">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G41" s="78" t="str" cm="1">
+      <c r="G41" s="77" t="str" cm="1">
         <f t="array" ref="G41">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -11925,7 +11920,7 @@
         <f t="array" ref="F42">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G42" s="78" t="str" cm="1">
+      <c r="G42" s="77" t="str" cm="1">
         <f t="array" ref="G42">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -11943,7 +11938,7 @@
         <f t="array" ref="F43">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G43" s="78" t="str" cm="1">
+      <c r="G43" s="77" t="str" cm="1">
         <f t="array" ref="G43">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -11961,7 +11956,7 @@
         <f t="array" ref="F44">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G44" s="78" t="str" cm="1">
+      <c r="G44" s="77" t="str" cm="1">
         <f t="array" ref="G44">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -11979,7 +11974,7 @@
         <f t="array" ref="F45">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="G45" s="78" t="str" cm="1">
+      <c r="G45" s="77" t="str" cm="1">
         <f t="array" ref="G45">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>NGAF 2025 Table 19</v>
       </c>
@@ -11997,7 +11992,7 @@
         <f t="array" ref="F46">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G46" s="78" t="str" cm="1">
+      <c r="G46" s="77" t="str" cm="1">
         <f t="array" ref="G46">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -12015,7 +12010,7 @@
         <f t="array" ref="F47">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G47" s="78" t="str" cm="1">
+      <c r="G47" s="77" t="str" cm="1">
         <f t="array" ref="G47">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -12033,7 +12028,7 @@
         <f t="array" ref="F48">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G48" s="78" t="str" cm="1">
+      <c r="G48" s="77" t="str" cm="1">
         <f t="array" ref="G48">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -12055,7 +12050,7 @@
         <f t="array" ref="F49">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G49" s="78" t="str" cm="1">
+      <c r="G49" s="77" t="str" cm="1">
         <f t="array" ref="G49">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
@@ -12073,7 +12068,7 @@
         <f t="array" ref="F50">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>
-      <c r="G50" s="78" t="str" cm="1">
+      <c r="G50" s="77" t="str" cm="1">
         <f t="array" ref="G50">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
single cell cell references updated to use name instead of cell reference
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v02.xlsx
+++ b/Excel/10_SolidWaste_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E5D735-7B3F-4223-9154-4EF731663506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369BC253-AE2C-453D-BE4A-A9E9DBFA16FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12645" firstSheet="1" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1350" yWindow="360" windowWidth="36255" windowHeight="19140" firstSheet="1" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -179,6 +179,7 @@
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variable">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.";"Fixed typo - Changed 'Fry' to 'Dry'."}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="Common_SourceData_DensityOfMethane_Data">'Constants - Common'!$D$175</definedName>
     <definedName name="CommonCropping_SourceData.CommonCropping_SourceData_FracGASFfInorganicFertiliser_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Fertiliser type f","FracGASFf","Basis";"Urea-based fertilisers",0.15,"Urea";"Ammonium-based fertilisers",0.08,"Ammonium";"Nitrate-based fertilisers",0.01,"Nitrate";"Ammonium-nitrate based fertilisers",0.05,"Ammonium-nitrate";"Other fertilisers",0.11,"Other"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="CommonCropping_SourceData.CommonCropping_SourceData_FracGASFfInorganicFertiliser_NIRReference">_xlfn.LAMBDA("IPCC 2019 Refinement Volume 4 Table 11.3 [1, p. 11]")</definedName>
     <definedName name="CommonCropping_SourceData.CommonCropping_SourceData_FracGASFfInorganicFertiliser_Source">_xlfn.LAMBDA("VEERG 2026:Table 12.2.2.9")</definedName>
@@ -16332,26 +16333,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -16546,30 +16527,31 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIAAnAEYAcgB5ACcAIAB0AG8AIAAnAEQAcgB5ACcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMgAwADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAZQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAVAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBQACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARQBUACAAPQAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZQB2AGEAcABvAHQAcgBhAG4AcwBwAGkAcgBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAATQBBAFQAIABtAGkAbgAgAGEAbgBkACAATQBBAFQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBlAGQAaQBhAG4AIABBAG4AbgB1AGEAbAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgACgATQBBAFQAKQBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBUAFwAIgAsACAAXAAiAE0AYQB4ACAATQBBAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIgADIANgAgAEMAXAAiACwAIAAyADYALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAXAAiADEANQAgAC0AIAAyADUAIABDAFwAIgAsACAAMQA1ACwAIAAyADUALgA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiIAAxADQAIABDAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQA0AC4AOQA5ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAFoAbwBuAGUAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIAA+ACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAD4AowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgACcAQQBxAHUAYQBjAHUAbAB0AHUAcgBlACcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQAnACwAIAAnAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAJwAgAGEAbgBkACAAJwBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAJwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlACcAIAByAG8AdwAgAHcAaQB0AGgAIABzAGEAbQBlACAARQBGACAAZgBvAHIAIABsAG8AdwAgAGEAbgBkACAAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBcAG4AVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcAG4ASQBQAEMAQwA6ACAATgAyAE8AIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABNAEEATgBBAEcARQBEACAAUwBPAEkATABTACwAIABBAE4ARAAgAEMATwAyACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATABJAE0ARQAgAEEATgBEACAAVQBSAEUAQQAgAEEAUABQAEwASQBDAEEAVABJAE8ATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAVwBFAFQAIABmAG8AcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBQAEMAQwAgADIAMAAxADkAIABSAGUAZgBpAG4AZQBtAGUAbgB0ACAAVgBvAGwAdQBtAGUAIAA0ADoAIABDAGgAYQBwAHQAZQByACAAMQAxADoAIABOADIATwAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAE0AYQBuAGEAZwBlAGQAIABTAG8AaQBsAHMALAAgAGEAbgBkACAAQwBPADIAIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABMAGkAbQBlACAAYQBuAGQAIABVAHIAZQBhACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAIABpAHIAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHAAcgBpAG4AawBsAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQByAGYAYQBjAGUAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAFQAYQBiAGwAZQAgAGMAcgBlAGEAdABlAGQAIABiAGEAcwBlAGQAIABvAG4AIABWAEUARQBSAEcAIAB0AGUAeAB0ACAAJwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgAnAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAnACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlACcAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBvAG4AdABoAHMAIAB0AG8AIABTAGUAYQBzAG8AbgBzACAATQBhAHAAcABpAG4AZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwBuAHQAaABcACIALAAgAFwAIgBTAGUAYQBzAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBhAG4AdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGIAcgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAcgBjAGgAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcAByAGkAbABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHkAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBuAGUAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBsAHkAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBnAHUAcwB0AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAcAB0AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwBjAHQAbwBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHYAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAYwBlAG0AYgBlAHIAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgABMgIABNAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAcABlAHIAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADgALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADIALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBcACIALAAgAFwAIgBNAEEAVAAgACgAugBDACkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBDAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIATABpAHEAdQBpAGQAIABTAGwAdQByAHIAeQAgACgAdwBpAHQAaABvAHUAdAAgAG4AYQB0AHUAcgBhAGwAIABjAHIAdQBzAHQAKQBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgACgAYgApAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAFMAdABvAHIAYQBnAGUAIAA8ADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAJwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAZQBwAGEAcgBhAHQAZQAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAAQQBkAGQAZQBkACAAJwBNAEEAVAAgAHIAYQB3ACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBpAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMQAuADQAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIAAmACAAXAAiACAAXAAiACAAJgAgAFQAaQB0AGwAZQBDAGUAbABsAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEAOgAgAFcAYQBzAHQAZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQAwAC4AMQAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAFMAbwBsAGkAZAAgAFcAYQBzAHQAZQAgAFQAcgBlAGEAdABtAGUAbgB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4ARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdwBhAHMAdABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAGIAeQAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcAG4ARQBfAGcAXABuAHQAIABDAE8AMgBlAFwAbgBFAF8AZwA9AFwAXABzAHUAbQBfAHQAXABcAHMAdQBtAF8AdwAoAFEAXwB3AHQAXABcAHQAaQBtAGUAcwAgAEUARgBfAHcAdABnACkAXABuAFEAXwB3AHQAIAA9ACAAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAbwBmACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACwAIABvAG4AIABhACAAdwBlAHQAIAB3AGUAaQBnAGgAdAAgAGIAYQBzAGkAcwAgACgAdAApAFwAbgBFAEYAXwB3AHQAZwAgAD0AIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAZwAgAGYAbwByACAAdABoAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAbwBmACAAdwBhAHMAdABlACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACAAKAB0ACAAQwBPADIAZQAvAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwB3AHQALAAgAEUARgBfAHcAdABnACwAXABuACAAIAAgACAAUQBfAHcAdAAgACoAIABFAEYAXwB3AHQAZwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMQAwAC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB0AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdwAoAFEAXwB7AHcAdAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AHcAdABnAH0AKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAXAAiACwAIABcACIAdABcACIALAAgAFwAIgBTAHUAbQAgAG8AZgAgAFEAXwB2AG8AbAB3AHQAIABhAG4AZAAgAFEAXwBtAGEAcwBzAHcAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AdwB0AGcAXAAiACwAIABcACIAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgB0ACAAQwBPADIAZQAvAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB3AFwAIgAsACAAXAAiAHcAYQBzAHQAZQAgAHQAeQBwAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB0AFwAIgAsACAAXAAiAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAZwBcACIALAAgAFwAIgBnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AdgBvAGwAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGQAIAB3AGEAcwB0AGUAIABpAG4AcAB1AHQAIABhAHMAIAB2AG8AbAB1AG0AZQAgAGEAbgBkACAAYwBvAG4AdgBlAHIAdABlAGQAIAB0AG8AIAB0AG8AbgBuAGUAcwBcACIALAAgAFwAIgB0AG8AbgBuAGUAcwBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADEAMAAuADEALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AbQBhAHMAcwB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAbQBhAHMAcwBcACIALAAgAFwAIgB0AG8AbgBuAGUAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFEAXwB2AG8AbAB3AHQAIABhAG4AZAAgAFEAXwBtAGEAcwBzAHcAdAAgAHYAYQByAGkAYQBiAGwAZQBzACAAdABvACAAYwBsAGUAYQByAGwAeQAgAHQAcgBhAGMAawAgAGkAbgBwAHUAdAAgAG8AcgAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABRACAAdgBhAGwAdQBlAHMAXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBcAG4ATQBhAHMAcwAgAG8AZgAgAHcAYQBzAHQAZQAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIAB2AG8AbAB1AG0AZQBcAG4AUQBfAHcAdABcAG4AdABcAG4AUQBfAHcAdAA9AFYAXwB3AHQAXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcAG4AVgBfAHcAdAAgAD0AIAB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAbQAzACkAXABuAFYAVABNAF8AdwAgAD0AIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABvAGYAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABmAG8AcgAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAKAB0AC8AbQAzACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVgBfAHcAdAAsACAAVgBUAE0AXwB3ACwAXABuACAAIAAgACAAVgBfAHcAdAAgACoAIABWAFQATQBfAHcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHMAcwAgAG8AZgAgAHcAYQBzAHQAZQAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIAB2AG8AbAB1AG0AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB3AHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMQAwAC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUQBfAHsAdwB0AH0APQBWAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAAVgBUAE0AXwB3AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAF8AdwB0AFwAIgAsACAAXAAiAHYAbwBsAHUAbQBlACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0AFwAIgAsACAAXAAiAG0AMwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAVABNAF8AdwBcACIALAAgAFwAIgBjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABvAGYAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABmAG8AcgAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAHQALwBtADMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB3AFwAIgAsACAAXAAiAHcAYQBzAHQAZQAgAHQAeQBwAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB0AFwAIgAsACAAXAAiAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdwBhAHMAdABlAHMAIABkAGkAcwBwAG8AcwBlAGQAIABvAGYAIABhAHQAIABkAGkAZgBmAGUAcgBlAG4AdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdABpAGUAcwBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdwBhAHMAdABlAHMAIABkAGkAcwBwAG8AcwBlAGQAIABvAGYAIABhAHQAIABkAGkAZgBmAGUAcgBlAG4AdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdABpAGUAcwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAEYAdwB0AFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFUAbgBpAHQAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgB0ACAAQwBPADIAZQAgAC8AIAB0AFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAxAC4AMQBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMANQAsACAANAAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHQAeQBwAGUAIAB0AFwAIgAsACAAXAAiAFcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAEUARgB3AHQAXAAiACwAIABcACIARQBGACAAcwBvAHUAcgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADIALgAxACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAzAC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgA3ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADIALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADQALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUgB1AGIAYgBlAHIAIABhAG4AZAAgAGwAZQBhAHQAaABlAHIAXAAiACwAIAAzAC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG4AcwB0AHIAdQBjAHQAaQBvAG4AIABhAG4AZAAgAGQAZQBtAG8AbABpAHQAaQBvAG4AIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAsACAAZwByAGUAZQBuACAAdwBhAHMAdABlACwAIAB3AG8AbwBkACwAIABzAGwAdQBkAGcAZQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAAxADYAOQAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADAALgAzADYANgA3ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUgB1AGIAYgBlAHIAIABhAG4AZAAgAGwAZQBhAHQAaABlAHIAXAAiACwAIAAwAC4ANAA5ADEAOQAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAuADEAMQAwADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAwADUAMwA3ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgA2ADQAOQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcACIALAAgADAALgAwADQANgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAnAHAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAYgBvAGEAcgBkACcAIAB0AG8AIAAnAHAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAJwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAJwBwAHIAdQBuAG4AaQBuAGcAcwAnACAAdABvACAAJwBwAHIAdQBuAGkAbgBnAHMAJwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABFAEYAIABzAG8AdQByAGMAZQAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAcABlAGMAaQBmAGkAYwAgAHIAZQBmAGUAcgBlAG4AYwBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIAAnAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuADoAIABGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlACcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBDAG8AbQBwAG8AcwB0AGkAbgBnADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAJwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIAAnAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AOgAgAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQAnACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAOgAgAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwAgACgAdAAvAG0AMwApACAAKABWAFQATQB3ACkAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBUAE0AdwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgB0AC8AbQAzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADIALAAgADIALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAVgBUAE0AdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4ANQAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAuADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMQA1ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADcAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAuADQAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG4AcwB0AHIAdQBjAHQAaQBvAG4AIABhAG4AZAAgAGQAZQBtAG8AbABpAHQAaQBvAG4AIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA5AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBoAGEAbgBnAGUAZAAgAGMAbwBsAHUAbQBuACAAaABlAGEAZABlAHIAIABDAEYAdwAgAHQAbwAgAFYAVABNAHcAIAB0AG8AIABtAGEAdABjAGgAIAB0AGkAdABsAGUAIAB2AGEAcgBpAGEAYgBsAGUALgBcACIAKQApADsAXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsACAAVwBhAHMAdABlAFQAeQBwAGUALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABVAG4AaQB0AFQAeQBwAGUALABcAG4AIAAgAFMAVQBNAEkARgBTACgAXABuACAAIAAgACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAXABuACAAIAAgACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFwAbgAgACAAIAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABVAG4AaQB0AFQAeQBwAGUAXABuACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0ACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16588,6 +16570,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
scope 3 build scripts
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v02.xlsx
+++ b/Excel/10_SolidWaste_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C41BB7-87A2-4C93-8CE7-53CBEB51F2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86BFCC9-2004-4AC4-8ED0-C0707B322240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="36255" windowHeight="19140" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -21,9 +21,6 @@
     <sheet name="Constants - Solid Waste" sheetId="110" r:id="rId6"/>
     <sheet name="Constants - Common" sheetId="124" r:id="rId7"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId8"/>
-  </externalReferences>
   <definedNames>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -278,21 +275,13 @@
     <definedName name="WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume_Unit">_xlfn.LAMBDA("t")</definedName>
     <definedName name="WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume_Variable">_xlfn.LAMBDA("Q_wt")</definedName>
     <definedName name="WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment">_xlfn.LAMBDA(_xlpm.TreatmentArray,_xlpm.WasteArray,_xlpm.TreatmentLocationArray,_xlpm.UnitArray,_xlpm.AmountArray,_xlpm.TreatmentType,_xlpm.WasteType,_xlpm.TreatmentLocationType,_xlpm.UnitType, SUMIFS(_xlpm.AmountArray, _xlpm.TreatmentArray, _xlpm.TreatmentType, _xlpm.WasteArray, _xlpm.WasteType, _xlpm.TreatmentLocationArray, _xlpm.TreatmentLocationType, _xlpm.UnitArray, _xlpm.UnitType))</definedName>
-    <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data">_xlfn.LAMBDA(
-  _xlfn.MAKEARRAY(35, 4,
-    _xlfn.LAMBDA(_xlpm.r,_xlpm.c,
-      INDEX({"Treatment type t","Waste type w","EFwt","EF source";"Landfill","Food waste (including animal carcasses, spoiled animal feed or crop)",2.1,"NGAF 2025 table 15";"Landfill","Paper and cardboard",3.3,"NGAF 2025 table 15";"Landfill","Green waste (including crop residues or prunings)",1.6,"NGAF 2025 table 15";"Landfill","Wood",0.7,"NGAF 2025 table 15";"Landfill","Textiles",2,"NGAF 2025 table 15";"Landfill","Sludge",0.4,"NGAF 2025 table 15";"Landfill","Rubber and leather",3.3,"NGAF 2025 table 15";"Landfill","Inert waste (including concrete, metal, plastic or glass)",0,"NGAF 2025 table 15";"Landfill","Municipal solid waste",1.6,"NGAF 2025 table 15";"Landfill","Commercial and industrial waste",1.3,"NGAF 2025 table 15";"Landfill","Construction and demolition waste",0.2,"NGAF 2025 table 15";"Incineration","Food waste, green waste, wood, sludge",0,"";"Incineration","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Incineration","Green waste (including crop residues or prunings)","","";"Incineration","Wood","","";"Incineration","Sludge","","";"Incineration","Paper and cardboard",0.0169,"";"Incineration","Textiles",0.3667,"";"Incineration","Rubber and leather",0.4919,"";"Incineration","Inert waste (including concrete, metal, plastic or glass)",0.11,"";"Incineration","Municipal solid waste",0.0537,"NGAF 2025 Table 18";"Incineration","Commercial and industrial waste",1.649,"NGAF 2025 Table 18";"Composting","All organic waste",0.046,"NGAF 2025 Table 19";"Composting","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Composting","Green waste (including crop residues or prunings)","","";"Composting","Wood","","";"Composting","Sludge","","";"Composting","Paper and cardboard","","";"Anaerobic digestion","All organic waste",0.028,"NGAF 2025 Table 19";"Anaerobic digestion","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Anaerobic digestion","Green waste (including crop residues or prunings)","","";"Anaerobic digestion","Wood","","";"Anaerobic digestion","Sludge","","";"Anaerobic digestion","Paper and cardboard","",""}, _xlpm.r, _xlpm.c)
-)))</definedName>
+    <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(35, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Treatment type t","Waste type w","EFwt","EF source";"Landfill","Food waste (including animal carcasses, spoiled animal feed or crop)",2.1,"NGAF 2025 table 15";"Landfill","Paper and cardboard",3.3,"NGAF 2025 table 15";"Landfill","Green waste (including crop residues or prunings)",1.6,"NGAF 2025 table 15";"Landfill","Wood",0.7,"NGAF 2025 table 15";"Landfill","Textiles",2,"NGAF 2025 table 15";"Landfill","Sludge",0.4,"NGAF 2025 table 15";"Landfill","Rubber and leather",3.3,"NGAF 2025 table 15";"Landfill","Inert waste (including concrete, metal, plastic or glass)",0,"NGAF 2025 table 15";"Landfill","Municipal solid waste",1.6,"NGAF 2025 table 15";"Landfill","Commercial and industrial waste",1.3,"NGAF 2025 table 15";"Landfill","Construction and demolition waste",0.2,"NGAF 2025 table 15";"Incineration","Food waste, green waste, wood, sludge",0,"";"Incineration","Food waste (including animal carcasses, spoiled animal feed or crop)",0,"";"Incineration","Green waste (including crop residues or prunings)",0,"";"Incineration","Wood",0,"";"Incineration","Sludge",0,"";"Incineration","Paper and cardboard",0.0169,"";"Incineration","Textiles",0.3667,"";"Incineration","Rubber and leather",0.4919,"";"Incineration","Inert waste (including concrete, metal, plastic or glass)",0.11,"";"Incineration","Municipal solid waste",0.0537,"NGAF 2025 Table 18";"Incineration","Commercial and industrial waste",1.649,"NGAF 2025 Table 18";"Composting","All organic waste",0.046,"NGAF 2025 Table 19";"Composting","Food waste (including animal carcasses, spoiled animal feed or crop)",0.046,"";"Composting","Green waste (including crop residues or prunings)",0.046,"";"Composting","Wood",0.046,"";"Composting","Sludge",0.046,"";"Composting","Paper and cardboard",0.046,"";"Anaerobic digestion","All organic waste",0.028,"NGAF 2025 Table 19";"Anaerobic digestion","Food waste (including animal carcasses, spoiled animal feed or crop)",0.028,"";"Anaerobic digestion","Green waste (including crop residues or prunings)",0.028,"";"Anaerobic digestion","Wood",0.028,"";"Anaerobic digestion","Sludge",0.028,"";"Anaerobic digestion","Paper and cardboard",0.028,""}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Source">_xlfn.LAMBDA(("VEERG 2026: Table A.4.1.1"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Title">_xlfn.LAMBDA(("Emission factors for wastes disposed of at different treatment facilities"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Unit">_xlfn.LAMBDA(("t CO2e / t"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Variable">_xlfn.LAMBDA(("EFwt"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(7, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION ON SOURCE:";"Fixed typo 'paper and carboard' to 'paper and cardboard'";"Fixed typo 'prunnings' to 'prunings'";"Added EF source column with specific references";"Added sub-categories for 'Incineration: Food waste, green waste, wood, sludge' in order to use volume to mass conversion factor values";"Added sub-categories for 'Composting: All organic waste' in order to use volume to mass conversion factor values";"Added sub-categories for 'Anaerobic digestion: All organic waste' in order to use volume to mass conversion factor values"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data">_xlfn.LAMBDA(
-  _xlfn.MAKEARRAY(12, 2,
-    _xlfn.LAMBDA(_xlpm.r,_xlpm.c,
-      INDEX({"Waste type w","VTMw";"Food waste (including animal carcasses, spoiled animal feed or crop)",0.5;"Paper and cardboard",0.09;"Green waste (including crop residues or prunings)",0.24;"Wood",0.15;"Textiles",0.14;"Sludge",0.72;"Rubber and leather",0.14;"Inert waste (including concrete, metal, plastic or glass)",0.42;"Municipal solid waste",0.36;"Commercial and industrial waste",0.33;"Construction and demolition waste",0.39}, _xlpm.r, _xlpm.c)
-)))</definedName>
+    <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(12, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Waste type w","VTMw";"Food waste (including animal carcasses, spoiled animal feed or crop)",0.5;"Paper and cardboard",0.09;"Green waste (including crop residues or prunings)",0.24;"Wood",0.15;"Textiles",0.14;"Sludge",0.72;"Rubber and leather",0.14;"Inert waste (including concrete, metal, plastic or glass)",0.42;"Municipal solid waste",0.36;"Commercial and industrial waste",0.33;"Construction and demolition waste",0.39}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Source">_xlfn.LAMBDA(("VEERG 2026: Table A.4.1.2"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Title">_xlfn.LAMBDA(("Volume to mass conversion factor for various waste types"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Unit">_xlfn.LAMBDA(("t/m3"))</definedName>
@@ -2103,6 +2092,176 @@
   <dxfs count="74">
     <dxf>
       <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2967,176 +3126,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -3588,8 +3577,8 @@
     <mruColors>
       <color rgb="FF0C769E"/>
       <color rgb="FF008000"/>
+      <color rgb="FFCC6600"/>
       <color rgb="FFFFCCCC"/>
-      <color rgb="FFCC6600"/>
       <color rgb="FFC44340"/>
       <color rgb="FF183C1B"/>
       <color rgb="FFDCECD0"/>
@@ -4391,26 +4380,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Home"/>
-      <sheetName val="Constants - Common"/>
-      <sheetName val="Acknowledgements"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -4569,49 +4538,49 @@
     <tableColumn id="1" xr3:uid="{4BCCA81B-E068-42CD-9919-4775D49C0C4A}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{799E3DE8-DD14-4DCE-B966-842CD3CF53AF}" name="MAT" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{799E3DE8-DD14-4DCE-B966-842CD3CF53AF}" name="MAT" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{C2288789-DCFC-48C9-A709-62081E5498A6}" name="MAP" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{C2288789-DCFC-48C9-A709-62081E5498A6}" name="MAP" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{017A9A14-BC38-49CF-82DD-1E74C23C473A}" name="Frost days per year" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{017A9A14-BC38-49CF-82DD-1E74C23C473A}" name="Frost days per year" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{FFC28617-1BCE-4686-BA60-3CBBD2DBDED6}" name="Elevation" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{FFC28617-1BCE-4686-BA60-3CBBD2DBDED6}" name="Elevation" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{AB8020AC-D2A8-458E-AC2C-05752C6978AF}" name="MAP:PET" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{AB8020AC-D2A8-458E-AC2C-05752C6978AF}" name="MAP:PET" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{232818F5-1E5C-4F21-9AF1-99D3361FB313}" name="Min temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{232818F5-1E5C-4F21-9AF1-99D3361FB313}" name="Min temp" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{9D529497-E48F-4AD1-A52B-A6AFC9977A99}" name="Max temp" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{9D529497-E48F-4AD1-A52B-A6AFC9977A99}" name="Max temp" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{D634F9C4-7AA1-4B28-8927-4B35F6B3C6D2}" name="Min rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{D634F9C4-7AA1-4B28-8927-4B35F6B3C6D2}" name="Min rainfall" totalsRowDxfId="45" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{22C210E1-3964-49A8-ABCA-85AE06650916}" name="Max rainfall" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{22C210E1-3964-49A8-ABCA-85AE06650916}" name="Max rainfall" totalsRowDxfId="44" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{99862E90-4C38-4030-9B0C-B4010DAA753C}" name="Min frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{99862E90-4C38-4030-9B0C-B4010DAA753C}" name="Min frost days" totalsRowDxfId="43" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{49F2E192-6E79-47C1-B3E8-0A9974D7AFE7}" name="Max frost days" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{49F2E192-6E79-47C1-B3E8-0A9974D7AFE7}" name="Max frost days" totalsRowDxfId="42" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4D1C8B6E-5909-42FD-8D3A-7396B1656514}" name="Min elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{4D1C8B6E-5909-42FD-8D3A-7396B1656514}" name="Min elevation" totalsRowDxfId="41" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{42A57023-BA2E-4A74-A523-1601325D53F7}" name="Max elevation" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{42A57023-BA2E-4A74-A523-1601325D53F7}" name="Max elevation" totalsRowDxfId="40" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{D10E3032-4D1E-46DD-B901-2DE6E69812EA}" name="Min MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{D10E3032-4D1E-46DD-B901-2DE6E69812EA}" name="Min MAP:PET" totalsRowDxfId="39" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{CF785213-3CBC-485C-89BA-E0FEDD22E926}" name="Max MAP:PET" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{CF785213-3CBC-485C-89BA-E0FEDD22E926}" name="Max MAP:PET" totalsRowDxfId="38" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4629,7 +4598,7 @@
     <tableColumn id="1" xr3:uid="{7540654D-96F8-46F3-B26C-7976EC8EC4A4}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1B5500D9-B94B-4112-BBF5-102D84360327}" name="Wet or Dry Zone" totalsRowDxfId="20" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{1B5500D9-B94B-4112-BBF5-102D84360327}" name="Wet or Dry Zone" totalsRowDxfId="37" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4735,7 +4704,7 @@
     <tableColumn id="1" xr3:uid="{A09175F0-2A84-4DAD-86F1-85B060C78212}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{BF611C02-A3C7-4C2F-BCF7-C7161F309936}" name="FracWET" dataDxfId="19">
+    <tableColumn id="2" xr3:uid="{BF611C02-A3C7-4C2F-BCF7-C7161F309936}" name="FracWET" dataDxfId="36">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4809,7 +4778,7 @@
     <tableColumn id="1" xr3:uid="{0205EB41-8BF3-4501-A595-2D4A7C50BFE1}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{359F335D-C699-47FC-848D-C87C57DFCDC2}" name="FracWET" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{359F335D-C699-47FC-848D-C87C57DFCDC2}" name="FracWET" dataDxfId="35" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4827,7 +4796,7 @@
     <tableColumn id="1" xr3:uid="{60C1796B-E277-4D1C-BC5D-4BA32A8A69EC}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0BE8B7EC-26F1-4120-A0D6-9BE10AE79E7F}" name="EFPRP" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{0BE8B7EC-26F1-4120-A0D6-9BE10AE79E7F}" name="EFPRP" dataDxfId="34" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4845,7 +4814,7 @@
     <tableColumn id="1" xr3:uid="{F5B5661A-F22C-4325-B84D-F2494578C60D}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A506AFB5-E9EE-42C0-AE4D-7CBC0FFAA059}" name="Season" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{A506AFB5-E9EE-42C0-AE4D-7CBC0FFAA059}" name="Season" dataDxfId="33" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4877,49 +4846,49 @@
     <tableColumn id="1" xr3:uid="{0188288F-977B-49E5-80CC-FB92F6326B64}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{76097606-F5E4-4513-84C2-1E3E9502A474}" name="MAT (ºC)" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{76097606-F5E4-4513-84C2-1E3E9502A474}" name="MAT (ºC)" dataDxfId="32" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{CCB8C26B-443C-46D4-8EDC-7351295ABBDB}" name="Anaerobic lagoon" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{CCB8C26B-443C-46D4-8EDC-7351295ABBDB}" name="Anaerobic lagoon" dataDxfId="31" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{19DC7330-9B62-4895-8F67-A4D4CAA24028}" name="Digester / covered lagoons" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{19DC7330-9B62-4895-8F67-A4D4CAA24028}" name="Digester / covered lagoons" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{6391496C-B15D-44D9-A952-82348BBD76E2}" name="Liquid systems" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{6391496C-B15D-44D9-A952-82348BBD76E2}" name="Liquid systems" dataDxfId="29" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{9B478D0D-7DE8-4A56-8246-338C8FC0E7ED}" name="Daily spread" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{9B478D0D-7DE8-4A56-8246-338C8FC0E7ED}" name="Daily spread" dataDxfId="28" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D2FD97A5-3214-4AD2-B8CF-2D2B56AC9BBA}" name="Composting (passive windrow)" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{D2FD97A5-3214-4AD2-B8CF-2D2B56AC9BBA}" name="Composting (passive windrow)" dataDxfId="27" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0A3D6F37-43C1-4178-B30A-1F643BCDA688}" name="Solid storage" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{0A3D6F37-43C1-4178-B30A-1F643BCDA688}" name="Solid storage" dataDxfId="26" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5CA08DAF-0BB0-4256-AC81-CD5D7E55E7B6}" name="Pit storage" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{5CA08DAF-0BB0-4256-AC81-CD5D7E55E7B6}" name="Pit storage" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{22353178-A4F9-46F4-80A3-8568FCEC1C99}" name="Deep litter" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{22353178-A4F9-46F4-80A3-8568FCEC1C99}" name="Deep litter" dataDxfId="24" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D06C2DD5-D366-4EBD-B040-B999BCE76A03}" name="Poultry manure with bedding" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{D06C2DD5-D366-4EBD-B040-B999BCE76A03}" name="Poultry manure with bedding" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{F4051E78-BDEA-4B06-A255-6717B6AAD286}" name="Poultry manure without bedding" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{F4051E78-BDEA-4B06-A255-6717B6AAD286}" name="Poultry manure without bedding" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{24C138BB-96B7-487F-AB0F-7AB5E5EB4392}" name="Direct processing" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{24C138BB-96B7-487F-AB0F-7AB5E5EB4392}" name="Direct processing" dataDxfId="21" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{1EE4056F-863B-4CD5-909A-CF69E38FD6E4}" name="Direct application" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{1EE4056F-863B-4CD5-909A-CF69E38FD6E4}" name="Direct application" dataDxfId="20" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{A7F11F4F-12AF-462B-B803-34690706AE95}" name="Pasture range and paddock" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{A7F11F4F-12AF-462B-B803-34690706AE95}" name="Pasture range and paddock" dataDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{2105F6CB-9025-4A4B-AFCB-0EB6730C9F01}" name="MAT raw" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{2105F6CB-9025-4A4B-AFCB-0EB6730C9F01}" name="MAT raw" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4937,7 +4906,7 @@
     <tableColumn id="1" xr3:uid="{F76C5DCF-44F1-4BBB-8278-E3F8DAFD498E}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C4089206-0C91-4E29-A689-CD565DCAB189}" name="EFNi &amp; EFN2Oi" dataDxfId="0" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{C4089206-0C91-4E29-A689-CD565DCAB189}" name="EFNi &amp; EFN2Oi" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5278,7 +5247,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="803" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="838" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -5310,6 +5279,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53CF26AA-F4FA-460F-9B3A-C19960195F0B}">
+  <sheetPr>
+    <tabColor rgb="FF0C769E"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -5325,6 +5297,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D37CA77B-B50B-428D-99FC-773BB70E61A6}">
+  <sheetPr>
+    <tabColor rgb="FF0C769E"/>
+  </sheetPr>
   <dimension ref="A1:W45"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5532,6 +5507,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DE30AE0-5101-4331-B8DF-043DE9AAFBA8}">
   <sheetPr>
+    <tabColor rgb="FF0C769E"/>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
   <dimension ref="A1:H87"/>
@@ -6327,6 +6303,9 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC610A2-02A7-4F78-A2BB-B4DFE856D1FB}">
+  <sheetPr>
+    <tabColor theme="5" tint="-0.249977111117893"/>
+  </sheetPr>
   <dimension ref="A1:L385"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7093,87 +7072,87 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F162:F163">
-    <cfRule type="cellIs" dxfId="52" priority="20" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="20" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F174:F175">
-    <cfRule type="cellIs" dxfId="51" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="15" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F186:F187">
-    <cfRule type="cellIs" dxfId="50" priority="18" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="18" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F274:F275">
-    <cfRule type="cellIs" dxfId="49" priority="93" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="93" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F279:F280">
-    <cfRule type="cellIs" dxfId="48" priority="92" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="92" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F284:F285">
-    <cfRule type="cellIs" dxfId="47" priority="91" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="91" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F308:F309">
-    <cfRule type="cellIs" dxfId="46" priority="85" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="85" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F313:F314">
-    <cfRule type="cellIs" dxfId="45" priority="84" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="84" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F318:F319">
-    <cfRule type="cellIs" dxfId="44" priority="83" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="83" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I33 F71">
-    <cfRule type="cellIs" dxfId="43" priority="62" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="62" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I79:I83">
-    <cfRule type="cellIs" dxfId="42" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I87 I146">
-    <cfRule type="cellIs" dxfId="41" priority="74" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="74" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I98:I100">
-    <cfRule type="cellIs" dxfId="40" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I104:I107">
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I111:I115">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J8 I65:I66 H67:H69 I68 I70:I72 I74:I75 I226 I232 E234:G234">
-    <cfRule type="cellIs" dxfId="37" priority="79" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="79" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J37 I59 F150:F151">
-    <cfRule type="cellIs" dxfId="36" priority="21" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="21" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7216,6 +7195,9 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEFC1CB6-2463-438A-90A4-6F54247DF8D8}">
+  <sheetPr>
+    <tabColor rgb="FF008000"/>
+  </sheetPr>
   <dimension ref="A1:L342"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -11176,6 +11158,9 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84A5A36D-67BF-491B-8BEC-65303FBC20AD}">
+  <sheetPr>
+    <tabColor theme="2" tint="-0.499984740745262"/>
+  </sheetPr>
   <dimension ref="A1:AI165"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -11733,9 +11718,9 @@
         <f t="array" ref="E29">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Food waste (including animal carcasses, spoiled animal feed or crop)</v>
       </c>
-      <c r="F29" s="26" t="str" cm="1">
+      <c r="F29" s="26" cm="1">
         <f t="array" ref="F29">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G29" s="26" t="str" cm="1">
         <f t="array" ref="G29">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -11751,9 +11736,9 @@
         <f t="array" ref="E30">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Green waste (including crop residues or prunings)</v>
       </c>
-      <c r="F30" s="26" t="str" cm="1">
+      <c r="F30" s="26" cm="1">
         <f t="array" ref="F30">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G30" s="26" t="str" cm="1">
         <f t="array" ref="G30">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -11769,9 +11754,9 @@
         <f t="array" ref="E31">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Wood</v>
       </c>
-      <c r="F31" s="26" t="str" cm="1">
+      <c r="F31" s="26" cm="1">
         <f t="array" ref="F31">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G31" s="26" t="str" cm="1">
         <f t="array" ref="G31">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -11787,9 +11772,9 @@
         <f t="array" ref="E32">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Sludge</v>
       </c>
-      <c r="F32" s="26" t="str" cm="1">
+      <c r="F32" s="26" cm="1">
         <f t="array" ref="F32">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G32" s="26" t="str" cm="1">
         <f t="array" ref="G32">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -11931,9 +11916,9 @@
         <f t="array" ref="E40">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Food waste (including animal carcasses, spoiled animal feed or crop)</v>
       </c>
-      <c r="F40" s="26" t="str" cm="1">
+      <c r="F40" s="26" cm="1">
         <f t="array" ref="F40">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="G40" s="77" t="str" cm="1">
         <f t="array" ref="G40">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -11949,9 +11934,9 @@
         <f t="array" ref="E41">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Green waste (including crop residues or prunings)</v>
       </c>
-      <c r="F41" s="26" t="str" cm="1">
+      <c r="F41" s="26" cm="1">
         <f t="array" ref="F41">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="G41" s="77" t="str" cm="1">
         <f t="array" ref="G41">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -11967,9 +11952,9 @@
         <f t="array" ref="E42">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Wood</v>
       </c>
-      <c r="F42" s="26" t="str" cm="1">
+      <c r="F42" s="26" cm="1">
         <f t="array" ref="F42">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="G42" s="77" t="str" cm="1">
         <f t="array" ref="G42">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -11985,9 +11970,9 @@
         <f t="array" ref="E43">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Sludge</v>
       </c>
-      <c r="F43" s="26" t="str" cm="1">
+      <c r="F43" s="26" cm="1">
         <f t="array" ref="F43">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="G43" s="77" t="str" cm="1">
         <f t="array" ref="G43">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -12003,9 +11988,9 @@
         <f t="array" ref="E44">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Paper and cardboard</v>
       </c>
-      <c r="F44" s="26" t="str" cm="1">
+      <c r="F44" s="26" cm="1">
         <f t="array" ref="F44">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="G44" s="77" t="str" cm="1">
         <f t="array" ref="G44">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -12039,9 +12024,9 @@
         <f t="array" ref="E46">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Food waste (including animal carcasses, spoiled animal feed or crop)</v>
       </c>
-      <c r="F46" s="26" t="str" cm="1">
+      <c r="F46" s="26" cm="1">
         <f t="array" ref="F46">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="G46" s="77" t="str" cm="1">
         <f t="array" ref="G46">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -12057,9 +12042,9 @@
         <f t="array" ref="E47">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Green waste (including crop residues or prunings)</v>
       </c>
-      <c r="F47" s="26" t="str" cm="1">
+      <c r="F47" s="26" cm="1">
         <f t="array" ref="F47">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="G47" s="77" t="str" cm="1">
         <f t="array" ref="G47">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -12075,9 +12060,9 @@
         <f t="array" ref="E48">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Wood</v>
       </c>
-      <c r="F48" s="26" t="str" cm="1">
+      <c r="F48" s="26" cm="1">
         <f t="array" ref="F48">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="G48" s="77" t="str" cm="1">
         <f t="array" ref="G48">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -12097,9 +12082,9 @@
         <f t="array" ref="E49">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Sludge</v>
       </c>
-      <c r="F49" s="26" t="str" cm="1">
+      <c r="F49" s="26" cm="1">
         <f t="array" ref="F49">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="G49" s="77" t="str" cm="1">
         <f t="array" ref="G49">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -12115,9 +12100,9 @@
         <f t="array" ref="E50">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
         <v>Paper and cardboard</v>
       </c>
-      <c r="F50" s="26" t="str" cm="1">
+      <c r="F50" s="26" cm="1">
         <f t="array" ref="F50">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v/>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="G50" s="77" t="str" cm="1">
         <f t="array" ref="G50">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -12392,6 +12377,9 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFAEEE30-F12E-424A-B51D-10898C859B82}">
+  <sheetPr>
+    <tabColor theme="2" tint="-0.499984740745262"/>
+  </sheetPr>
   <dimension ref="A1:BY259"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -16383,26 +16371,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -16597,30 +16565,31 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxADoAIABXAGEAcwB0AGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AbABpAGQAIABXAGEAcwB0AGUAIABUAHIAZQBhAHQAbQBlAG4AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXABuAEUAXwBnAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAGcAPQBcAFwAcwB1AG0AXwB0AFwAXABzAHUAbQBfAHcAKABRAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB3AHQAZwApAFwAbgBRAF8AdwB0ACAAPQAgAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAIAAoAHQAKQBcAG4ARQBGAF8AdwB0AGcAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAdAAgAEMATwAyAGUALwB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AdwB0ACwAIABFAEYAXwB3AHQAZwAsAFwAbgAgACAAIAAgAFEAXwB3AHQAIAAqACAARQBGAF8AdwB0AGcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdABcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHcAKABRAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewB3AHQAZwB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzAFwAIgAsACAAXAAiAHQAXAAiACwAIABcACIAUwB1AG0AIABvAGYAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAHcAdABnAFwAIgAsACAAXAAiAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAdAAgAEMATwAyAGUALwB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGcAXAAiACwAIABcACIAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHYAbwBsAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAdgBvAGwAdQBtAGUAIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAdABvAG4AbgBlAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAxADAALgAxAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAG0AYQBzAHMAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AYQBzAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAIAB2AGEAcgBpAGEAYgBsAGUAcwAgAHQAbwAgAGMAbABlAGEAcgBsAHkAIAB0AHIAYQBjAGsAIABpAG4AcAB1AHQAIABvAHIAIABjAGEAbABjAHUAbABhAHQAZQBkACAAUQAgAHYAYQBsAHUAZQBzAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXABuAFEAXwB3AHQAXABuAHQAXABuAFEAXwB3AHQAPQBWAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXABuAFYAXwB3AHQAIAA9ACAAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAG0AMwApAFwAbgBWAFQATQBfAHcAIAA9ACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgACgAdAAvAG0AMwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAXwB3AHQALAAgAFYAVABNAF8AdwAsAFwAbgAgACAAIAAgAFYAXwB3AHQAIAAqACAAVgBUAE0AXwB3AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AdwB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB7AHcAdAB9AD0AVgBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBfAHcAdABcACIALAAgAFwAIgB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgBtADMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFQATQBfAHcAXAAiACwAIABcACIAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgB0AC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBGAHcAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAgAEMATwAyAGUAIAAvACAAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADEAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzADUALAAgADQALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIAB0AHkAcABlACAAdABcACIALAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBFAEYAdwB0AFwAIgAsACAAXAAiAEUARgAgAHMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAyAC4AMQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4ANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAyAC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA0ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUALAAgAGcAcgBlAGUAbgAgAHcAYQBzAHQAZQAsACAAdwBvAG8AZAAsACAAcwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMQA2ADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMwA2ADYANwAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADQAOQAxADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgAxADEAMAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA1ADMANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgA0ADkALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAAxACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAXAB1ADAAMAAyADcAcABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBiAG8AYQByAGQAXAB1ADAAMAAyADcAIAB0AG8AIABcAHUAMAAwADIANwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAdQAwADAAMgA3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABcAHUAMAAwADIANwBwAHIAdQBuAG4AaQBuAGcAcwBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AHAAcgB1AG4AaQBuAGcAcwBcAHUAMAAwADIANwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABFAEYAIABzAG8AdQByAGMAZQAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAcABlAGMAaQBmAGkAYwAgAHIAZQBmAGUAcgBlAG4AYwBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgA6ACAARgBvAG8AZAAgAHcAYQBzAHQAZQAsACAAZwByAGUAZQBuACAAdwBhAHMAdABlACwAIAB3AG8AbwBkACwAIABzAGwAdQBkAGcAZQBcAHUAMAAwADIANwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBDAG8AbQBwAG8AcwB0AGkAbgBnADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAB1ADAAMAAyADcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAXAB1ADAAMAAyADcAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgA6ACAAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAdQAwADAAMgA3ACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAOgAgAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwAgACgAdAAvAG0AMwApACAAKABWAFQATQB3ACkAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBUAE0AdwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgB0AC8AbQAzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADIALAAgADIALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAVgBUAE0AdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4ANQAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAuADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMQA1ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADcAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAuADQAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG4AcwB0AHIAdQBjAHQAaQBvAG4AIABhAG4AZAAgAGQAZQBtAG8AbABpAHQAaQBvAG4AIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA5AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBoAGEAbgBnAGUAZAAgAGMAbwBsAHUAbQBuACAAaABlAGEAZABlAHIAIABDAEYAdwAgAHQAbwAgAFYAVABNAHcAIAB0AG8AIABtAGEAdABjAGgAIAB0AGkAdABsAGUAIAB2AGEAcgBpAGEAYgBsAGUALgBcACIAKQApADsAXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsACAAVwBhAHMAdABlAFQAeQBwAGUALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABVAG4AaQB0AFQAeQBwAGUALABcAG4AIAAgAFMAVQBNAEkARgBTACgAXABuACAAIAAgACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAXABuACAAIAAgACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFwAbgAgACAAIAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABVAG4AaQB0AFQAeQBwAGUAXABuACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0ACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIAAnAEYAcgB5ACcAIAB0AG8AIAAnAEQAcgB5ACcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMgAwADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAZQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAVAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBQACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARQBUACAAPQAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZQB2AGEAcABvAHQAcgBhAG4AcwBwAGkAcgBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAATQBBAFQAIABtAGkAbgAgAGEAbgBkACAATQBBAFQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBlAGQAaQBhAG4AIABBAG4AbgB1AGEAbAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgACgATQBBAFQAKQBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBUAFwAIgAsACAAXAAiAE0AYQB4ACAATQBBAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIgADIANgAgAEMAXAAiACwAIAAyADYALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAXAAiADEANQAgAC0AIAAyADUAIABDAFwAIgAsACAAMQA1ACwAIAAyADUALgA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiIAAxADQAIABDAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQA0AC4AOQA5ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAFoAbwBuAGUAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIAA+ACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAD4AowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgACcAQQBxAHUAYQBjAHUAbAB0AHUAcgBlACcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQAnACwAIAAnAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAJwAgAGEAbgBkACAAJwBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAJwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlACcAIAByAG8AdwAgAHcAaQB0AGgAIABzAGEAbQBlACAARQBGACAAZgBvAHIAIABsAG8AdwAgAGEAbgBkACAAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBcAG4AVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcAG4ASQBQAEMAQwA6ACAATgAyAE8AIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABNAEEATgBBAEcARQBEACAAUwBPAEkATABTACwAIABBAE4ARAAgAEMATwAyACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATABJAE0ARQAgAEEATgBEACAAVQBSAEUAQQAgAEEAUABQAEwASQBDAEEAVABJAE8ATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAVwBFAFQAIABmAG8AcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBQAEMAQwAgADIAMAAxADkAIABSAGUAZgBpAG4AZQBtAGUAbgB0ACAAVgBvAGwAdQBtAGUAIAA0ADoAIABDAGgAYQBwAHQAZQByACAAMQAxADoAIABOADIATwAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAE0AYQBuAGEAZwBlAGQAIABTAG8AaQBsAHMALAAgAGEAbgBkACAAQwBPADIAIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABMAGkAbQBlACAAYQBuAGQAIABVAHIAZQBhACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAIABpAHIAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHAAcgBpAG4AawBsAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQByAGYAYQBjAGUAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAFQAYQBiAGwAZQAgAGMAcgBlAGEAdABlAGQAIABiAGEAcwBlAGQAIABvAG4AIABWAEUARQBSAEcAIAB0AGUAeAB0ACAAJwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgAnAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAnACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlACcAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBvAG4AdABoAHMAIAB0AG8AIABTAGUAYQBzAG8AbgBzACAATQBhAHAAcABpAG4AZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwBuAHQAaABcACIALAAgAFwAIgBTAGUAYQBzAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBhAG4AdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGIAcgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAcgBjAGgAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcAByAGkAbABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHkAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBuAGUAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBsAHkAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBnAHUAcwB0AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAcAB0AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwBjAHQAbwBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHYAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAYwBlAG0AYgBlAHIAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgABMgIABNAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAcABlAHIAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADgALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADIALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBcACIALAAgAFwAIgBNAEEAVAAgACgAugBDACkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBDAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIATABpAHEAdQBpAGQAIABTAGwAdQByAHIAeQAgACgAdwBpAHQAaABvAHUAdAAgAG4AYQB0AHUAcgBhAGwAIABjAHIAdQBzAHQAKQBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgACgAYgApAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAFMAdABvAHIAYQBnAGUAIAA8ADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAJwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAZQBwAGEAcgBhAHQAZQAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAAQQBkAGQAZQBkACAAJwBNAEEAVAAgAHIAYQB3ACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBpAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMQAuADQAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgACYAIABcACIAIABcACIAIAAmACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQAwAC4AMQA6ACAAVwBhAHMAdABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAAUwBvAGwAaQBkACAAVwBhAHMAdABlACAAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAbgBFAF8AZwBcAG4AdAAgAEMATwAyAGUAXABuAEUAXwBnAD0AXABcAHMAdQBtAF8AdABcAFwAcwB1AG0AXwB3ACgAUQBfAHcAdABcAFwAdABpAG0AZQBzACAARQBGAF8AdwB0AGcAKQBcAG4AUQBfAHcAdAAgAD0AIABxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzACAAKAB0ACkAXABuAEUARgBfAHcAdABnACAAPQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAHQAIABDAE8AMgBlAC8AdAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUQBfAHcAdAAsACAARQBGAF8AdwB0AGcALABcAG4AIAAgACAAIABRAF8AdwB0ACAAKgAgAEUARgBfAHcAdABnAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdwBhAHMAdABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAGIAeQAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAPQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHQAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB3ACgAUQBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAdwB0AGcAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAbwBmACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACwAIABvAG4AIABhACAAdwBlAHQAIAB3AGUAaQBnAGgAdAAgAGIAYQBzAGkAcwBcACIALAAgAFwAIgB0AFwAIgAsACAAXAAiAFMAdQBtACAAbwBmACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwB3AHQAZwBcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAZwAgAGYAbwByACAAdABoAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAbwBmACAAdwBhAHMAdABlACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0AFwAIgAsACAAXAAiAHQAIABDAE8AMgBlAC8AdABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB2AG8AbAB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAHYAbwBsAHUAbQBlACAAYQBuAGQAIABjAG8AbgB2AGUAcgB0AGUAZAAgAHQAbwAgAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMQAwAC4AMQAuADEALgAxACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwBtAGEAcwBzAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABpAG4AcAB1AHQAIABhAHMAIABtAGEAcwBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0ACAAdgBhAHIAaQBhAGIAbABlAHMAIAB0AG8AIABjAGwAZQBhAHIAbAB5ACAAdAByAGEAYwBrACAAaQBuAHAAdQB0ACAAbwByACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAFEAIAB2AGEAbAB1AGUAcwBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAbgBRAF8AdwB0AFwAbgB0AFwAbgBRAF8AdwB0AD0AVgBfAHcAdABcAFwAdABpAG0AZQBzACAAVgBUAE0AXwB3AFwAbgBWAF8AdwB0ACAAPQAgAHYAbwBsAHUAbQBlACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACAAKABtADMAKQBcAG4AVgBUAE0AXwB3ACAAPQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIAAoAHQALwBtADMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAF8AdwB0ACwAIABWAFQATQBfAHcALABcAG4AIAAgACAAIABWAF8AdwB0ACAAKgAgAFYAVABNAF8AdwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUQBfAHcAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AewB3AHQAfQA9AFYAXwB7AHcAdAB9AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAXwB3AHQAXAAiACwAIABcACIAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAbQAzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBUAE0AXwB3AFwAIgAsACAAXAAiAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAdAAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUARgB3AHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQAIABDAE8AMgBlACAALwAgAHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAxAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwA1ACwAIAA0ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAdAB5AHAAZQAgAHQAXAAiACwAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIARQBGAHcAdABcACIALAAgAFwAIgBFAEYAIABzAG8AdQByAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMgAuADEALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAxAC4ANgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADcALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMgAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4ANAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBDAG8AbgBzAHQAcgB1AGMAdABpAG8AbgAgAGEAbgBkACAAZABlAG0AbwBsAGkAdABpAG8AbgAgAHcAYQBzAHQAZQBcACIALAAgADAALgAyACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADEANgA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADMANgA2ADcALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgA0ADkAMQA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwAC4AMQAxADAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANQAzADcALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYANAA5ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADgAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAAxACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAJwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZAAnACAAdABvACAAJwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkACcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgACcAcAByAHUAbgBuAGkAbgBnAHMAJwAgAHQAbwAgACcAcAByAHUAbgBpAG4AZwBzACcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAARQBGACAAcwBvAHUAcgBjAGUAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAHAAZQBjAGkAZgBpAGMAIAByAGUAZgBlAHIAZQBuAGMAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgA6ACAARgBvAG8AZAAgAHcAYQBzAHQAZQAsACAAZwByAGUAZQBuACAAdwBhAHMAdABlACwAIAB3AG8AbwBkACwAIABzAGwAdQBkAGcAZQAnACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgACcAQwBvAG0AcABvAHMAdABpAG4AZwA6ACAAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlACcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAJwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyADoAIABWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAIAAoAHQALwBtADMAKQAgACgAVgBUAE0AdwApAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAVABNAHcAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAvAG0AMwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAxAC4AMgBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAyACwAIAAyACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAFYAVABNAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAuADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA5ADsAXABuACAAIAAgACAAIAAgACAAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA3ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgA0ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADYAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAOQBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEMAaABhAG4AZwBlAGQAIABjAG8AbAB1AG0AbgAgAGgAZQBhAGQAZQByACAAQwBGAHcAIAB0AG8AIABWAFQATQB3ACAAdABvACAAbQBhAHQAYwBoACAAdABpAHQAbABlACAAdgBhAHIAaQBhAGIAbABlAC4AXAAiACkAKQA7AFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAVQBuAGkAdABUAHkAcABlACwAXABuACAAIABTAFUATQBJAEYAUwAoAFwAbgAgACAAIAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALABcAG4AIAAgACAAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABcAG4AIAAgACAAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAVQBuAGkAdABUAHkAcABlAFwAbgAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdAAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16639,6 +16608,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat(scripts): add find-errors checker; skip in-cell-image rich values and hide broken-fn library LAMBDAs by default
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v02.xlsx
+++ b/Excel/10_SolidWaste_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4680EFA3-9520-4E8C-92C0-77E528AF96A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3514BB3-F655-4EC9-AA9A-C269CECC94EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="2145" yWindow="2460" windowWidth="36255" windowHeight="19140" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -234,23 +234,6 @@
     <definedName name="Fertiliser_Equations_Lime.VEERG_5_3_1_1__1_LimeApplication">_xlfn.LAMBDA(_xlpm.Mlime,_xlpm.FracLime,_xlpm.Plime,_xlpm.EFlime,_xlpm.FracDol,_xlpm.Pdol,_xlpm.EFdol,_xlpm.CgCO2, ((_xlpm.Mlime * _xlpm.FracLime * _xlpm.Plime * _xlpm.EFlime) + (_xlpm.Mlime * _xlpm.FracDol * _xlpm.Pdol * _xlpm.EFdol)) * _xlpm.CgCO2 * 10 ^ -3)</definedName>
     <definedName name="Fertiliser_Equations_Organic.VEERG_5_2_1_1__2_MassOfNitrogenInOrganicFertiliser">_xlfn.LAMBDA(_xlpm.Morganicjf,_xlpm.FNorganicf, _xlpm.Morganicjf * _xlpm.FNorganicf)</definedName>
     <definedName name="getOverlappingReportingCycles">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingStartMonth,_xlpm.ReportingStartDay, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, _xlpm.ReportingStartMonth, _xlpm.d, _xlpm.ReportingStartDay, _xlpm.A, _xlpm.S - 364, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (DATE(_xlpm.ya, _xlpm.m, _xlpm.d) &lt; _xlpm.A), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
-    <definedName name="Inoput_Cell_Livestock_antibiotics">#REF!</definedName>
-    <definedName name="Inoput_Cell_Livestockantibiotics">#REF!</definedName>
-    <definedName name="Input_Cell_CO2_for_carbonation">#REF!</definedName>
-    <definedName name="Input_Cell_CO2forcarbonation">#REF!</definedName>
-    <definedName name="Input_Cell_Livestock_antibiotics">#REF!</definedName>
-    <definedName name="Input_Cell_Livestock_tags">#REF!</definedName>
-    <definedName name="Input_Cell_LivestockAntibiotics">#REF!</definedName>
-    <definedName name="Input_Cell_Nylon_netting_for_horticulture">#REF!</definedName>
-    <definedName name="Input_Cell_Nylonnettingforhorticulture">#REF!</definedName>
-    <definedName name="Input_Cell_Pallets__Plastic">#REF!</definedName>
-    <definedName name="Input_Cell_Pallets__Wood">#REF!</definedName>
-    <definedName name="Input_Cell_Pallets_Plastic">#REF!</definedName>
-    <definedName name="Input_Cell_Pallets_Wood">#REF!</definedName>
-    <definedName name="Range_LivestockStartingValues">#REF!</definedName>
-    <definedName name="Step1">#REF!</definedName>
-    <definedName name="Step2">#REF!</definedName>
-    <definedName name="Step3">#REF!</definedName>
     <definedName name="Table_E_g_offsite">'10.1.1-2 Solid waste treatment'!$D$156:$E$190</definedName>
     <definedName name="Table_E_g_onsite">'10.1.1-2 Solid waste treatment'!$D$115:$E$149</definedName>
     <definedName name="Table_V_w_t_offsite">'10.1.1-2 Solid waste treatment'!$D$58:$E$92</definedName>
@@ -16519,19 +16502,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIAAnAEYAcgB5ACcAIAB0AG8AIAAnAEQAcgB5ACcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMgAwADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAZQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAVAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBQACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARQBUACAAPQAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZQB2AGEAcABvAHQAcgBhAG4AcwBwAGkAcgBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAATQBBAFQAIABtAGkAbgAgAGEAbgBkACAATQBBAFQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBlAGQAaQBhAG4AIABBAG4AbgB1AGEAbAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgACgATQBBAFQAKQBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBUAFwAIgAsACAAXAAiAE0AYQB4ACAATQBBAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIgADIANgAgAEMAXAAiACwAIAAyADYALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAXAAiADEANQAgAC0AIAAyADUAIABDAFwAIgAsACAAMQA1ACwAIAAyADUALgA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiIAAxADQAIABDAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQA0AC4AOQA5ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAFoAbwBuAGUAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIAA+ACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAD4AowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgACcAQQBxAHUAYQBjAHUAbAB0AHUAcgBlACcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQAnACwAIAAnAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAJwAgAGEAbgBkACAAJwBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAJwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlACcAIAByAG8AdwAgAHcAaQB0AGgAIABzAGEAbQBlACAARQBGACAAZgBvAHIAIABsAG8AdwAgAGEAbgBkACAAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBcAG4AVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcAG4ASQBQAEMAQwA6ACAATgAyAE8AIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABNAEEATgBBAEcARQBEACAAUwBPAEkATABTACwAIABBAE4ARAAgAEMATwAyACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATABJAE0ARQAgAEEATgBEACAAVQBSAEUAQQAgAEEAUABQAEwASQBDAEEAVABJAE8ATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAVwBFAFQAIABmAG8AcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBQAEMAQwAgADIAMAAxADkAIABSAGUAZgBpAG4AZQBtAGUAbgB0ACAAVgBvAGwAdQBtAGUAIAA0ADoAIABDAGgAYQBwAHQAZQByACAAMQAxADoAIABOADIATwAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAE0AYQBuAGEAZwBlAGQAIABTAG8AaQBsAHMALAAgAGEAbgBkACAAQwBPADIAIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABMAGkAbQBlACAAYQBuAGQAIABVAHIAZQBhACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAIABpAHIAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHAAcgBpAG4AawBsAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQByAGYAYQBjAGUAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAFQAYQBiAGwAZQAgAGMAcgBlAGEAdABlAGQAIABiAGEAcwBlAGQAIABvAG4AIABWAEUARQBSAEcAIAB0AGUAeAB0ACAAJwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgAnAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAnACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlACcAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBvAG4AdABoAHMAIAB0AG8AIABTAGUAYQBzAG8AbgBzACAATQBhAHAAcABpAG4AZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwBuAHQAaABcACIALAAgAFwAIgBTAGUAYQBzAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBhAG4AdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGIAcgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAcgBjAGgAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcAByAGkAbABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHkAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBuAGUAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBsAHkAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBnAHUAcwB0AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAcAB0AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwBjAHQAbwBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHYAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAYwBlAG0AYgBlAHIAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgABMgIABNAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAcABlAHIAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADgALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADIALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBcACIALAAgAFwAIgBNAEEAVAAgACgAugBDACkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBDAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIATABpAHEAdQBpAGQAIABTAGwAdQByAHIAeQAgACgAdwBpAHQAaABvAHUAdAAgAG4AYQB0AHUAcgBhAGwAIABjAHIAdQBzAHQAKQBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgACgAYgApAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAFMAdABvAHIAYQBnAGUAIAA8ADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAJwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAZQBwAGEAcgBhAHQAZQAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAAQQBkAGQAZQBkACAAJwBNAEEAVAAgAHIAYQB3ACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBpAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMQAuADQAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgACYAIABcACIAIABcACIAIAAmACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQAwAC4AMQA6ACAAVwBhAHMAdABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAAUwBvAGwAaQBkACAAVwBhAHMAdABlACAAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAbgBFAF8AZwBcAG4AdAAgAEMATwAyAGUAXABuAEUAXwBnAD0AXABcAHMAdQBtAF8AdABcAFwAcwB1AG0AXwB3ACgAUQBfAHcAdABcAFwAdABpAG0AZQBzACAARQBGAF8AdwB0AGcAKQBcAG4AUQBfAHcAdAAgAD0AIABxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzACAAKAB0ACkAXABuAEUARgBfAHcAdABnACAAPQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAHQAIABDAE8AMgBlAC8AdAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUQBfAHcAdAAsACAARQBGAF8AdwB0AGcALABcAG4AIAAgACAAIABRAF8AdwB0ACAAKgAgAEUARgBfAHcAdABnAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdwBhAHMAdABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAGIAeQAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAPQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHQAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB3ACgAUQBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAdwB0AGcAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAbwBmACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACwAIABvAG4AIABhACAAdwBlAHQAIAB3AGUAaQBnAGgAdAAgAGIAYQBzAGkAcwBcACIALAAgAFwAIgB0AFwAIgAsACAAXAAiAFMAdQBtACAAbwBmACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwB3AHQAZwBcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAZwAgAGYAbwByACAAdABoAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAbwBmACAAdwBhAHMAdABlACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0AFwAIgAsACAAXAAiAHQAIABDAE8AMgBlAC8AdABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB2AG8AbAB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAHYAbwBsAHUAbQBlACAAYQBuAGQAIABjAG8AbgB2AGUAcgB0AGUAZAAgAHQAbwAgAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMQAwAC4AMQAuADEALgAxACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwBtAGEAcwBzAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABpAG4AcAB1AHQAIABhAHMAIABtAGEAcwBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0ACAAdgBhAHIAaQBhAGIAbABlAHMAIAB0AG8AIABjAGwAZQBhAHIAbAB5ACAAdAByAGEAYwBrACAAaQBuAHAAdQB0ACAAbwByACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAFEAIAB2AGEAbAB1AGUAcwBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAbgBRAF8AdwB0AFwAbgB0AFwAbgBRAF8AdwB0AD0AVgBfAHcAdABcAFwAdABpAG0AZQBzACAAVgBUAE0AXwB3AFwAbgBWAF8AdwB0ACAAPQAgAHYAbwBsAHUAbQBlACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACAAKABtADMAKQBcAG4AVgBUAE0AXwB3ACAAPQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIAAoAHQALwBtADMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAF8AdwB0ACwAIABWAFQATQBfAHcALABcAG4AIAAgACAAIABWAF8AdwB0ACAAKgAgAFYAVABNAF8AdwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUQBfAHcAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AewB3AHQAfQA9AFYAXwB7AHcAdAB9AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAXwB3AHQAXAAiACwAIABcACIAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAbQAzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBUAE0AXwB3AFwAIgAsACAAXAAiAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAdAAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUARgB3AHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQAIABDAE8AMgBlACAALwAgAHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAxAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwA1ACwAIAA0ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAdAB5AHAAZQAgAHQAXAAiACwAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIARQBGAHcAdABcACIALAAgAFwAIgBFAEYAIABzAG8AdQByAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMgAuADEALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAxAC4ANgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADcALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMgAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4ANAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBDAG8AbgBzAHQAcgB1AGMAdABpAG8AbgAgAGEAbgBkACAAZABlAG0AbwBsAGkAdABpAG8AbgAgAHcAYQBzAHQAZQBcACIALAAgADAALgAyACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADEANgA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADMANgA2ADcALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgA0ADkAMQA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwAC4AMQAxADAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANQAzADcALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYANAA5ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADgAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAAxACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAJwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZAAnACAAdABvACAAJwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkACcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgACcAcAByAHUAbgBuAGkAbgBnAHMAJwAgAHQAbwAgACcAcAByAHUAbgBpAG4AZwBzACcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAARQBGACAAcwBvAHUAcgBjAGUAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAHAAZQBjAGkAZgBpAGMAIAByAGUAZgBlAHIAZQBuAGMAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgA6ACAARgBvAG8AZAAgAHcAYQBzAHQAZQAsACAAZwByAGUAZQBuACAAdwBhAHMAdABlACwAIAB3AG8AbwBkACwAIABzAGwAdQBkAGcAZQAnACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgACcAQwBvAG0AcABvAHMAdABpAG4AZwA6ACAAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlACcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAJwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyADoAIABWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAIAAoAHQALwBtADMAKQAgACgAVgBUAE0AdwApAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAVABNAHcAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAvAG0AMwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAxAC4AMgBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAyACwAIAAyACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAFYAVABNAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAuADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA5ADsAXABuACAAIAAgACAAIAAgACAAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA3ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgA0ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADYAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAOQBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEMAaABhAG4AZwBlAGQAIABjAG8AbAB1AG0AbgAgAGgAZQBhAGQAZQByACAAQwBGAHcAIAB0AG8AIABWAFQATQB3ACAAdABvACAAbQBhAHQAYwBoACAAdABpAHQAbABlACAAdgBhAHIAaQBhAGIAbABlAC4AXAAiACkAKQA7AFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAVQBuAGkAdABUAHkAcABlACwAXABuACAAIABTAFUATQBJAEYAUwAoAFwAbgAgACAAIAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALABcAG4AIAAgACAAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABcAG4AIAAgACAAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAVQBuAGkAdABUAHkAcABlAFwAbgAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdAAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -16726,6 +16696,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIAAnAEYAcgB5ACcAIAB0AG8AIAAnAEQAcgB5ACcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMgAwADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAZQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAVAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBQACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARQBUACAAPQAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZQB2AGEAcABvAHQAcgBhAG4AcwBwAGkAcgBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAATQBBAFQAIABtAGkAbgAgAGEAbgBkACAATQBBAFQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBlAGQAaQBhAG4AIABBAG4AbgB1AGEAbAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgACgATQBBAFQAKQBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBUAFwAIgAsACAAXAAiAE0AYQB4ACAATQBBAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIgADIANgAgAEMAXAAiACwAIAAyADYALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAXAAiADEANQAgAC0AIAAyADUAIABDAFwAIgAsACAAMQA1ACwAIAAyADUALgA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiIAAxADQAIABDAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQA0AC4AOQA5ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAFoAbwBuAGUAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIAA+ACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAD4AowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgACcAQQBxAHUAYQBjAHUAbAB0AHUAcgBlACcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQAnACwAIAAnAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAJwAgAGEAbgBkACAAJwBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAJwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlACcAIAByAG8AdwAgAHcAaQB0AGgAIABzAGEAbQBlACAARQBGACAAZgBvAHIAIABsAG8AdwAgAGEAbgBkACAAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBcAG4AVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcAG4ASQBQAEMAQwA6ACAATgAyAE8AIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABNAEEATgBBAEcARQBEACAAUwBPAEkATABTACwAIABBAE4ARAAgAEMATwAyACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATABJAE0ARQAgAEEATgBEACAAVQBSAEUAQQAgAEEAUABQAEwASQBDAEEAVABJAE8ATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAVwBFAFQAIABmAG8AcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBQAEMAQwAgADIAMAAxADkAIABSAGUAZgBpAG4AZQBtAGUAbgB0ACAAVgBvAGwAdQBtAGUAIAA0ADoAIABDAGgAYQBwAHQAZQByACAAMQAxADoAIABOADIATwAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAE0AYQBuAGEAZwBlAGQAIABTAG8AaQBsAHMALAAgAGEAbgBkACAAQwBPADIAIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABMAGkAbQBlACAAYQBuAGQAIABVAHIAZQBhACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAIABpAHIAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHAAcgBpAG4AawBsAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQByAGYAYQBjAGUAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAFQAYQBiAGwAZQAgAGMAcgBlAGEAdABlAGQAIABiAGEAcwBlAGQAIABvAG4AIABWAEUARQBSAEcAIAB0AGUAeAB0ACAAJwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgAnAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAnACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlACcAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBvAG4AdABoAHMAIAB0AG8AIABTAGUAYQBzAG8AbgBzACAATQBhAHAAcABpAG4AZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwBuAHQAaABcACIALAAgAFwAIgBTAGUAYQBzAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBhAG4AdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGIAcgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAcgBjAGgAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcAByAGkAbABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHkAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBuAGUAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBsAHkAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBnAHUAcwB0AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAcAB0AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwBjAHQAbwBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHYAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAYwBlAG0AYgBlAHIAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgABMgIABNAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAcABlAHIAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADgALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADIALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBcACIALAAgAFwAIgBNAEEAVAAgACgAugBDACkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBDAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIATABpAHEAdQBpAGQAIABTAGwAdQByAHIAeQAgACgAdwBpAHQAaABvAHUAdAAgAG4AYQB0AHUAcgBhAGwAIABjAHIAdQBzAHQAKQBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgACgAYgApAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAFMAdABvAHIAYQBnAGUAIAA8ADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAJwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAZQBwAGEAcgBhAHQAZQAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAAQQBkAGQAZQBkACAAJwBNAEEAVAAgAHIAYQB3ACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBpAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMQAuADQAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgACYAIABcACIAIABcACIAIAAmACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQAwAC4AMQA6ACAAVwBhAHMAdABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAAUwBvAGwAaQBkACAAVwBhAHMAdABlACAAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAbgBFAF8AZwBcAG4AdAAgAEMATwAyAGUAXABuAEUAXwBnAD0AXABcAHMAdQBtAF8AdABcAFwAcwB1AG0AXwB3ACgAUQBfAHcAdABcAFwAdABpAG0AZQBzACAARQBGAF8AdwB0AGcAKQBcAG4AUQBfAHcAdAAgAD0AIABxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzACAAKAB0ACkAXABuAEUARgBfAHcAdABnACAAPQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAHQAIABDAE8AMgBlAC8AdAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUQBfAHcAdAAsACAARQBGAF8AdwB0AGcALABcAG4AIAAgACAAIABRAF8AdwB0ACAAKgAgAEUARgBfAHcAdABnAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdwBhAHMAdABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAGIAeQAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAPQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHQAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB3ACgAUQBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAdwB0AGcAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAbwBmACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACwAIABvAG4AIABhACAAdwBlAHQAIAB3AGUAaQBnAGgAdAAgAGIAYQBzAGkAcwBcACIALAAgAFwAIgB0AFwAIgAsACAAXAAiAFMAdQBtACAAbwBmACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwB3AHQAZwBcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAZwAgAGYAbwByACAAdABoAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAbwBmACAAdwBhAHMAdABlACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0AFwAIgAsACAAXAAiAHQAIABDAE8AMgBlAC8AdABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB2AG8AbAB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAHYAbwBsAHUAbQBlACAAYQBuAGQAIABjAG8AbgB2AGUAcgB0AGUAZAAgAHQAbwAgAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMQAwAC4AMQAuADEALgAxACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwBtAGEAcwBzAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABpAG4AcAB1AHQAIABhAHMAIABtAGEAcwBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0ACAAdgBhAHIAaQBhAGIAbABlAHMAIAB0AG8AIABjAGwAZQBhAHIAbAB5ACAAdAByAGEAYwBrACAAaQBuAHAAdQB0ACAAbwByACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAFEAIAB2AGEAbAB1AGUAcwBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAbgBRAF8AdwB0AFwAbgB0AFwAbgBRAF8AdwB0AD0AVgBfAHcAdABcAFwAdABpAG0AZQBzACAAVgBUAE0AXwB3AFwAbgBWAF8AdwB0ACAAPQAgAHYAbwBsAHUAbQBlACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACAAKABtADMAKQBcAG4AVgBUAE0AXwB3ACAAPQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIAAoAHQALwBtADMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAF8AdwB0ACwAIABWAFQATQBfAHcALABcAG4AIAAgACAAIABWAF8AdwB0ACAAKgAgAFYAVABNAF8AdwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUQBfAHcAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AewB3AHQAfQA9AFYAXwB7AHcAdAB9AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAXwB3AHQAXAAiACwAIABcACIAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAbQAzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBUAE0AXwB3AFwAIgAsACAAXAAiAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAdAAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUARgB3AHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQAIABDAE8AMgBlACAALwAgAHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAxAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwA1ACwAIAA0ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAdAB5AHAAZQAgAHQAXAAiACwAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIARQBGAHcAdABcACIALAAgAFwAIgBFAEYAIABzAG8AdQByAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMgAuADEALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAxAC4ANgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADcALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMgAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4ANAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBDAG8AbgBzAHQAcgB1AGMAdABpAG8AbgAgAGEAbgBkACAAZABlAG0AbwBsAGkAdABpAG8AbgAgAHcAYQBzAHQAZQBcACIALAAgADAALgAyACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADEANgA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADMANgA2ADcALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgA0ADkAMQA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwAC4AMQAxADAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANQAzADcALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYANAA5ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADgAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAAxACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAJwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZAAnACAAdABvACAAJwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkACcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgACcAcAByAHUAbgBuAGkAbgBnAHMAJwAgAHQAbwAgACcAcAByAHUAbgBpAG4AZwBzACcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAARQBGACAAcwBvAHUAcgBjAGUAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAHAAZQBjAGkAZgBpAGMAIAByAGUAZgBlAHIAZQBuAGMAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgA6ACAARgBvAG8AZAAgAHcAYQBzAHQAZQAsACAAZwByAGUAZQBuACAAdwBhAHMAdABlACwAIAB3AG8AbwBkACwAIABzAGwAdQBkAGcAZQAnACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgACcAQwBvAG0AcABvAHMAdABpAG4AZwA6ACAAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlACcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAJwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyADoAIABWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAIAAoAHQALwBtADMAKQAgACgAVgBUAE0AdwApAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAVABNAHcAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAvAG0AMwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAxAC4AMgBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAyACwAIAAyACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAFYAVABNAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAuADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA5ADsAXABuACAAIAAgACAAIAAgACAAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA3ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgA0ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADYAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAOQBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEMAaABhAG4AZwBlAGQAIABjAG8AbAB1AG0AbgAgAGgAZQBhAGQAZQByACAAQwBGAHcAIAB0AG8AIABWAFQATQB3ACAAdABvACAAbQBhAHQAYwBoACAAdABpAHQAbABlACAAdgBhAHIAaQBhAGIAbABlAC4AXAAiACkAKQA7AFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAVQBuAGkAdABUAHkAcABlACwAXABuACAAIABTAFUATQBJAEYAUwAoAFwAbgAgACAAIAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALABcAG4AIAAgACAAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABcAG4AIAAgACAAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAVQBuAGkAdABUAHkAcABlAFwAbgAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdAAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -16738,22 +16721,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16772,6 +16739,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
add sum function error checking
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v02.xlsx
+++ b/Excel/10_SolidWaste_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3514BB3-F655-4EC9-AA9A-C269CECC94EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF24E753-6096-43A3-ACF8-2C790B187381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2145" yWindow="2460" windowWidth="36255" windowHeight="19140" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="615" yWindow="2460" windowWidth="37785" windowHeight="19140" firstSheet="4" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -2235,169 +2235,11 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
         <family val="2"/>
         <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <family val="2"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -3257,11 +3099,169 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
         <family val="2"/>
         <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <family val="2"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -4502,49 +4502,49 @@
     <tableColumn id="1" xr3:uid="{41AD31C2-222E-4203-AB79-4AE1B7722F01}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{CF7EC01F-AE07-49E9-9441-45922CBE6114}" name="MAT" totalsRowDxfId="61" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{CF7EC01F-AE07-49E9-9441-45922CBE6114}" name="MAT" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{581BABDE-82D6-446A-9071-BCA1C1E40BC3}" name="MAP" totalsRowDxfId="60" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{581BABDE-82D6-446A-9071-BCA1C1E40BC3}" name="MAP" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{F34AC3E4-E53B-4604-A8DA-45DEF26A6E82}" name="Frost days per year" totalsRowDxfId="59" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{F34AC3E4-E53B-4604-A8DA-45DEF26A6E82}" name="Frost days per year" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0895F24E-AAD7-408E-B612-3D581AD80DF9}" name="Elevation" totalsRowDxfId="58" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{0895F24E-AAD7-408E-B612-3D581AD80DF9}" name="Elevation" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{918D7B00-0110-48E8-AD9C-D31724B4783E}" name="MAP:PET" totalsRowDxfId="57" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{918D7B00-0110-48E8-AD9C-D31724B4783E}" name="MAP:PET" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{68C8FAA3-A87C-4CBA-9853-85C1CB1597C6}" name="Min temp" totalsRowDxfId="56" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{68C8FAA3-A87C-4CBA-9853-85C1CB1597C6}" name="Min temp" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0EAD5DCC-C795-459A-8820-2C2E89D9C6B6}" name="Max temp" totalsRowDxfId="55" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{0EAD5DCC-C795-459A-8820-2C2E89D9C6B6}" name="Max temp" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{30FE0BAC-9697-4787-AEB0-75F9FCD5AE32}" name="Min rainfall" totalsRowDxfId="54" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{30FE0BAC-9697-4787-AEB0-75F9FCD5AE32}" name="Min rainfall" totalsRowDxfId="45" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{22609E04-F91A-4706-BF03-3A1821B04EFE}" name="Max rainfall" totalsRowDxfId="53" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{22609E04-F91A-4706-BF03-3A1821B04EFE}" name="Max rainfall" totalsRowDxfId="44" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{14F0DEEB-5FA1-4BD6-AE13-791D12D24F4F}" name="Min frost days" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{14F0DEEB-5FA1-4BD6-AE13-791D12D24F4F}" name="Min frost days" totalsRowDxfId="43" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{8ED18250-E62D-4810-B4D2-291CC16FA7F0}" name="Max frost days" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{8ED18250-E62D-4810-B4D2-291CC16FA7F0}" name="Max frost days" totalsRowDxfId="42" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{04556D12-4AB9-4892-8184-C215A2623153}" name="Min elevation" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{04556D12-4AB9-4892-8184-C215A2623153}" name="Min elevation" totalsRowDxfId="41" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{A31B38B1-BE7A-4AD4-AA00-DAF2EC3A9026}" name="Max elevation" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{A31B38B1-BE7A-4AD4-AA00-DAF2EC3A9026}" name="Max elevation" totalsRowDxfId="40" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{914D09DC-516A-4EC4-8695-330CAFAABEA4}" name="Min MAP:PET" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{914D09DC-516A-4EC4-8695-330CAFAABEA4}" name="Min MAP:PET" totalsRowDxfId="39" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{5309E391-9596-47A3-9F4E-A1D6B26C7C04}" name="Max MAP:PET" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{5309E391-9596-47A3-9F4E-A1D6B26C7C04}" name="Max MAP:PET" totalsRowDxfId="38" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4562,7 +4562,7 @@
     <tableColumn id="1" xr3:uid="{BD6A576D-B2B7-4D78-835E-4F61589A29B5}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DF111C20-3B8E-4130-B4C5-9202DB915746}" name="Wet or Dry Zone" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{DF111C20-3B8E-4130-B4C5-9202DB915746}" name="Wet or Dry Zone" totalsRowDxfId="37" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4668,7 +4668,7 @@
     <tableColumn id="1" xr3:uid="{45C7EEF5-2D76-432E-9AB3-2CCF20D96CC4}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{805D4875-B508-476D-9520-35538202DE62}" name="FracWET" dataDxfId="45">
+    <tableColumn id="2" xr3:uid="{805D4875-B508-476D-9520-35538202DE62}" name="FracWET" dataDxfId="36">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4718,13 +4718,13 @@
     <tableColumn id="1" xr3:uid="{27ECD0A0-9936-4A60-BCC5-02F0C62FDA6C}" name="Treatment type t">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B7AF1F5E-7BAC-4FF7-B59E-F905655514F2}" name="Waste type w" dataDxfId="25" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B7AF1F5E-7BAC-4FF7-B59E-F905655514F2}" name="Waste type w" dataDxfId="61" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{EEC6B364-DA50-41AA-A530-330FAEE98233}" name="EFwt" dataDxfId="24" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{EEC6B364-DA50-41AA-A530-330FAEE98233}" name="EFwt" dataDxfId="60" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{01FD94D2-85D3-4478-AB5E-04E4027C2978}" name="EF source" dataDxfId="23" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{01FD94D2-85D3-4478-AB5E-04E4027C2978}" name="EF source" dataDxfId="59" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4742,7 +4742,7 @@
     <tableColumn id="1" xr3:uid="{06C6CF89-0895-4496-B260-975EDDE66F43}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{65257743-5E74-4B22-91DB-3D2E171C0562}" name="FracWET" dataDxfId="44" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{65257743-5E74-4B22-91DB-3D2E171C0562}" name="FracWET" dataDxfId="35" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4760,7 +4760,7 @@
     <tableColumn id="1" xr3:uid="{D893B6C1-E916-4A7E-97C2-CF70CA9EA2AF}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{7BAD82A9-AE37-4590-805C-2B3CC2381C9A}" name="EFPRP" dataDxfId="43" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{7BAD82A9-AE37-4590-805C-2B3CC2381C9A}" name="EFPRP" dataDxfId="34" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4778,7 +4778,7 @@
     <tableColumn id="1" xr3:uid="{A1E87281-FD70-4777-BB64-21908A3B7A0F}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{45807656-3C84-4037-B0E3-29092D3B5AE1}" name="Season" dataDxfId="42" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{45807656-3C84-4037-B0E3-29092D3B5AE1}" name="Season" dataDxfId="33" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4810,49 +4810,49 @@
     <tableColumn id="1" xr3:uid="{966FFE72-1919-4001-A8C1-B50F1B327852}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2896456D-9798-47E1-B33D-42D3227E1C58}" name="MAT (ºC)" dataDxfId="41" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{2896456D-9798-47E1-B33D-42D3227E1C58}" name="MAT (ºC)" dataDxfId="32" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{39A17CE5-6B6E-432D-BB0F-E166785B3835}" name="Anaerobic lagoon" dataDxfId="40" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{39A17CE5-6B6E-432D-BB0F-E166785B3835}" name="Anaerobic lagoon" dataDxfId="31" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B746B36E-2DB9-4A5A-8ED5-3D01E7C27149}" name="Digester / covered lagoons" dataDxfId="39" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{B746B36E-2DB9-4A5A-8ED5-3D01E7C27149}" name="Digester / covered lagoons" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{C103677F-98E6-4B81-933E-782382272D67}" name="Liquid systems" dataDxfId="38" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{C103677F-98E6-4B81-933E-782382272D67}" name="Liquid systems" dataDxfId="29" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{35AF51F0-1F56-4071-87BF-55E630E50B10}" name="Daily spread" dataDxfId="37" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{35AF51F0-1F56-4071-87BF-55E630E50B10}" name="Daily spread" dataDxfId="28" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{8E182D3B-654F-4747-BB3F-DEDE497496B4}" name="Composting (passive windrow)" dataDxfId="36" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{8E182D3B-654F-4747-BB3F-DEDE497496B4}" name="Composting (passive windrow)" dataDxfId="27" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{269BD40D-F086-416B-A820-75F37ABA5198}" name="Solid storage" dataDxfId="35" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{269BD40D-F086-416B-A820-75F37ABA5198}" name="Solid storage" dataDxfId="26" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{FFCCBA77-4B2D-4A9B-A4F9-E5B3C667415D}" name="Pit storage" dataDxfId="34" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{FFCCBA77-4B2D-4A9B-A4F9-E5B3C667415D}" name="Pit storage" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{1FC5E424-F954-46A3-A7E2-BC4244A5275A}" name="Deep litter" dataDxfId="33" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{1FC5E424-F954-46A3-A7E2-BC4244A5275A}" name="Deep litter" dataDxfId="24" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{2844977C-EBF6-4837-B7A9-81D3A93457A4}" name="Poultry manure with bedding" dataDxfId="32" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{2844977C-EBF6-4837-B7A9-81D3A93457A4}" name="Poultry manure with bedding" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{A8150F46-62C5-4A43-A256-E9630EA71C79}" name="Poultry manure without bedding" dataDxfId="31" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{A8150F46-62C5-4A43-A256-E9630EA71C79}" name="Poultry manure without bedding" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{12036AC1-5946-4C80-A7A2-EE87D193F90F}" name="Direct processing" dataDxfId="30" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{12036AC1-5946-4C80-A7A2-EE87D193F90F}" name="Direct processing" dataDxfId="21" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{926A2153-745E-4EA9-8280-BF3B7E476FF1}" name="Direct application" dataDxfId="29" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{926A2153-745E-4EA9-8280-BF3B7E476FF1}" name="Direct application" dataDxfId="20" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{7391D537-6E9F-4FBE-99CC-39D278B4C8EA}" name="Pasture range and paddock" dataDxfId="28" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{7391D537-6E9F-4FBE-99CC-39D278B4C8EA}" name="Pasture range and paddock" dataDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{13CCB745-C5B3-4DFE-BD61-A4D02CA55182}" name="MAT raw" dataDxfId="27" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{13CCB745-C5B3-4DFE-BD61-A4D02CA55182}" name="MAT raw" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4870,7 +4870,7 @@
     <tableColumn id="1" xr3:uid="{3447C239-7AB2-4C34-A553-096ADC63C59F}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2712239C-E043-49D7-94AA-19C6C38B44B9}" name="EFNi &amp; EFN2Oi" dataDxfId="26" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{2712239C-E043-49D7-94AA-19C6C38B44B9}" name="EFNi &amp; EFN2Oi" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4888,7 +4888,7 @@
     <tableColumn id="1" xr3:uid="{E899A810-DA34-4DD3-9420-7017118A50BC}" name="Waste type w">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data(), Table_SourceData_WasteSolid_VolumeToMassConversion[[#Headers],[Waste type w]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EC8E9200-43B6-459C-B7A6-907C4A1A3CDE}" name="VTMw" dataDxfId="22" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{EC8E9200-43B6-459C-B7A6-907C4A1A3CDE}" name="VTMw" dataDxfId="58" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data(), Table_SourceData_WasteSolid_VolumeToMassConversion[[#Headers],[Waste type w]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4911,7 +4911,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}" name="Table_WasteTypes_Incineration" displayName="Table_WasteTypes_Incineration" ref="K16:K26" totalsRowShown="0" headerRowDxfId="21" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}" name="Table_WasteTypes_Incineration" displayName="Table_WasteTypes_Incineration" ref="K16:K26" totalsRowShown="0" headerRowDxfId="57" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="K16:K26" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
@@ -4925,12 +4925,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}" name="Table_WasteTypes_Composting" displayName="Table_WasteTypes_Composting" ref="M16:M21" totalsRowShown="0" headerRowDxfId="20" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}" name="Table_WasteTypes_Composting" displayName="Table_WasteTypes_Composting" ref="M16:M21" totalsRowShown="0" headerRowDxfId="56" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="M16:M21" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{5B9ABACD-52AE-4D64-BCA6-1DA86A1A3FC3}" name="Waste type w" totalsRowDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{5B9ABACD-52AE-4D64-BCA6-1DA86A1A3FC3}" name="Waste type w" totalsRowDxfId="55" dataCellStyle="Content normal">
       <calculatedColumnFormula>E40</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4939,12 +4939,12 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}" name="Table_WasteTypes_Anaerobicdigestion" displayName="Table_WasteTypes_Anaerobicdigestion" ref="O16:O21" totalsRowShown="0" headerRowDxfId="18" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}" name="Table_WasteTypes_Anaerobicdigestion" displayName="Table_WasteTypes_Anaerobicdigestion" ref="O16:O21" totalsRowShown="0" headerRowDxfId="54" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="O16:O21" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{2D7DB5DA-05BB-4621-B5A8-576415999BBC}" name="Waste type w" totalsRowDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{2D7DB5DA-05BB-4621-B5A8-576415999BBC}" name="Waste type w" totalsRowDxfId="53" dataCellStyle="Content normal">
       <calculatedColumnFormula>E46</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9428,7 +9428,7 @@
         <v>Not used</v>
       </c>
       <c r="I127" s="26">
-        <f>SUM(G128:G131)+SUM(H128:H131)</f>
+        <f>SUM(G128:G131)+SUM(H128:H131)+N("Partial sum")</f>
         <v>74</v>
       </c>
       <c r="J127" s="26" cm="1">
@@ -9561,7 +9561,7 @@
         <v>4.5</v>
       </c>
       <c r="I132" s="26">
-        <f t="shared" si="1"/>
+        <f>G132+H132+N("Partial sum")</f>
         <v>54.5</v>
       </c>
       <c r="J132" s="26" cm="1">
@@ -9734,7 +9734,7 @@
         <v>Not used</v>
       </c>
       <c r="I138" s="26">
-        <f>SUM(G139:G143)+SUM(H139:H143)</f>
+        <f>SUM(G139:G143)+SUM(H139:H143)+N("Partial sum")</f>
         <v>29.5</v>
       </c>
       <c r="J138" s="26" cm="1">
@@ -9892,7 +9892,7 @@
         <v>Not used</v>
       </c>
       <c r="I144" s="26">
-        <f>SUM(G145:G149)+SUM(H145:H149)</f>
+        <f>SUM(G145:G149)+SUM(H145:H149)+N("Partial sum")</f>
         <v>0</v>
       </c>
       <c r="J144" s="26" cm="1">
@@ -10421,7 +10421,7 @@
         <v>Not used</v>
       </c>
       <c r="I168" s="26">
-        <f>SUM(G169:G172)+SUM(H169:H172)</f>
+        <f>SUM(G169:G172)+SUM(H169:H172)+N("Partial sum")</f>
         <v>62</v>
       </c>
       <c r="J168" s="26" cm="1">
@@ -10727,7 +10727,7 @@
         <v>Not used</v>
       </c>
       <c r="I179" s="26">
-        <f>SUM(G180:G184)+SUM(H180:H184)</f>
+        <f>SUM(G180:G184)+SUM(H180:H184)+N("Partial sum")</f>
         <v>100</v>
       </c>
       <c r="J179" s="26" cm="1">
@@ -10885,7 +10885,7 @@
         <v>Not used</v>
       </c>
       <c r="I185" s="26">
-        <f>SUM(G186:G190)+SUM(H186:H190)</f>
+        <f>SUM(G186:G190)+SUM(H186:H190)+N("Partial sum")</f>
         <v>0</v>
       </c>
       <c r="J185" s="26" cm="1">
@@ -16502,6 +16502,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -16696,31 +16716,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIAAnAEYAcgB5ACcAIAB0AG8AIAAnAEQAcgB5ACcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMgAwADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAZQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAVAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBQACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARQBUACAAPQAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZQB2AGEAcABvAHQAcgBhAG4AcwBwAGkAcgBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAATQBBAFQAIABtAGkAbgAgAGEAbgBkACAATQBBAFQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBlAGQAaQBhAG4AIABBAG4AbgB1AGEAbAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgACgATQBBAFQAKQBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBUAFwAIgAsACAAXAAiAE0AYQB4ACAATQBBAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIgADIANgAgAEMAXAAiACwAIAAyADYALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAXAAiADEANQAgAC0AIAAyADUAIABDAFwAIgAsACAAMQA1ACwAIAAyADUALgA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiIAAxADQAIABDAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQA0AC4AOQA5ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAFoAbwBuAGUAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIAA+ACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAD4AowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgACcAQQBxAHUAYQBjAHUAbAB0AHUAcgBlACcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQAnACwAIAAnAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAJwAgAGEAbgBkACAAJwBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAJwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlACcAIAByAG8AdwAgAHcAaQB0AGgAIABzAGEAbQBlACAARQBGACAAZgBvAHIAIABsAG8AdwAgAGEAbgBkACAAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBcAG4AVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcAG4ASQBQAEMAQwA6ACAATgAyAE8AIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABNAEEATgBBAEcARQBEACAAUwBPAEkATABTACwAIABBAE4ARAAgAEMATwAyACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATABJAE0ARQAgAEEATgBEACAAVQBSAEUAQQAgAEEAUABQAEwASQBDAEEAVABJAE8ATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAVwBFAFQAIABmAG8AcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBQAEMAQwAgADIAMAAxADkAIABSAGUAZgBpAG4AZQBtAGUAbgB0ACAAVgBvAGwAdQBtAGUAIAA0ADoAIABDAGgAYQBwAHQAZQByACAAMQAxADoAIABOADIATwAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAE0AYQBuAGEAZwBlAGQAIABTAG8AaQBsAHMALAAgAGEAbgBkACAAQwBPADIAIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABMAGkAbQBlACAAYQBuAGQAIABVAHIAZQBhACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAIABpAHIAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHAAcgBpAG4AawBsAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQByAGYAYQBjAGUAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAFQAYQBiAGwAZQAgAGMAcgBlAGEAdABlAGQAIABiAGEAcwBlAGQAIABvAG4AIABWAEUARQBSAEcAIAB0AGUAeAB0ACAAJwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgAnAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAnACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlACcAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBvAG4AdABoAHMAIAB0AG8AIABTAGUAYQBzAG8AbgBzACAATQBhAHAAcABpAG4AZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwBuAHQAaABcACIALAAgAFwAIgBTAGUAYQBzAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBhAG4AdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGIAcgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAcgBjAGgAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcAByAGkAbABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHkAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBuAGUAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBsAHkAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBnAHUAcwB0AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAcAB0AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwBjAHQAbwBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHYAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAYwBlAG0AYgBlAHIAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgABMgIABNAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAcABlAHIAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADgALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADIALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBcACIALAAgAFwAIgBNAEEAVAAgACgAugBDACkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBDAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIATABpAHEAdQBpAGQAIABTAGwAdQByAHIAeQAgACgAdwBpAHQAaABvAHUAdAAgAG4AYQB0AHUAcgBhAGwAIABjAHIAdQBzAHQAKQBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgACgAYgApAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAFMAdABvAHIAYQBnAGUAIAA8ADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAJwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAZQBwAGEAcgBhAHQAZQAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAAQQBkAGQAZQBkACAAJwBNAEEAVAAgAHIAYQB3ACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBpAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMQAuADQAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgACYAIABcACIAIABcACIAIAAmACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQAwAC4AMQA6ACAAVwBhAHMAdABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAAUwBvAGwAaQBkACAAVwBhAHMAdABlACAAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAbgBFAF8AZwBcAG4AdAAgAEMATwAyAGUAXABuAEUAXwBnAD0AXABcAHMAdQBtAF8AdABcAFwAcwB1AG0AXwB3ACgAUQBfAHcAdABcAFwAdABpAG0AZQBzACAARQBGAF8AdwB0AGcAKQBcAG4AUQBfAHcAdAAgAD0AIABxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzACAAKAB0ACkAXABuAEUARgBfAHcAdABnACAAPQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAHQAIABDAE8AMgBlAC8AdAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUQBfAHcAdAAsACAARQBGAF8AdwB0AGcALABcAG4AIAAgACAAIABRAF8AdwB0ACAAKgAgAEUARgBfAHcAdABnAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdwBhAHMAdABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAGIAeQAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAPQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHQAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB3ACgAUQBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAdwB0AGcAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAbwBmACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACwAIABvAG4AIABhACAAdwBlAHQAIAB3AGUAaQBnAGgAdAAgAGIAYQBzAGkAcwBcACIALAAgAFwAIgB0AFwAIgAsACAAXAAiAFMAdQBtACAAbwBmACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwB3AHQAZwBcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAZwAgAGYAbwByACAAdABoAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAbwBmACAAdwBhAHMAdABlACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0AFwAIgAsACAAXAAiAHQAIABDAE8AMgBlAC8AdABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB2AG8AbAB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAHYAbwBsAHUAbQBlACAAYQBuAGQAIABjAG8AbgB2AGUAcgB0AGUAZAAgAHQAbwAgAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMQAwAC4AMQAuADEALgAxACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwBtAGEAcwBzAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABpAG4AcAB1AHQAIABhAHMAIABtAGEAcwBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0ACAAdgBhAHIAaQBhAGIAbABlAHMAIAB0AG8AIABjAGwAZQBhAHIAbAB5ACAAdAByAGEAYwBrACAAaQBuAHAAdQB0ACAAbwByACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAFEAIAB2AGEAbAB1AGUAcwBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAbgBRAF8AdwB0AFwAbgB0AFwAbgBRAF8AdwB0AD0AVgBfAHcAdABcAFwAdABpAG0AZQBzACAAVgBUAE0AXwB3AFwAbgBWAF8AdwB0ACAAPQAgAHYAbwBsAHUAbQBlACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACAAKABtADMAKQBcAG4AVgBUAE0AXwB3ACAAPQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIAAoAHQALwBtADMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAF8AdwB0ACwAIABWAFQATQBfAHcALABcAG4AIAAgACAAIABWAF8AdwB0ACAAKgAgAFYAVABNAF8AdwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUQBfAHcAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AewB3AHQAfQA9AFYAXwB7AHcAdAB9AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAXwB3AHQAXAAiACwAIABcACIAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAbQAzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBUAE0AXwB3AFwAIgAsACAAXAAiAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAdAAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUARgB3AHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQAIABDAE8AMgBlACAALwAgAHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAxAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwA1ACwAIAA0ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAdAB5AHAAZQAgAHQAXAAiACwAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIARQBGAHcAdABcACIALAAgAFwAIgBFAEYAIABzAG8AdQByAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMgAuADEALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAxAC4ANgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADcALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMgAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4ANAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBDAG8AbgBzAHQAcgB1AGMAdABpAG8AbgAgAGEAbgBkACAAZABlAG0AbwBsAGkAdABpAG8AbgAgAHcAYQBzAHQAZQBcACIALAAgADAALgAyACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADEANgA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADMANgA2ADcALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgA0ADkAMQA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwAC4AMQAxADAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANQAzADcALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYANAA5ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADgAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIAXAAiADsAXABuAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAAxACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAJwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZAAnACAAdABvACAAJwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkACcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgACcAcAByAHUAbgBuAGkAbgBnAHMAJwAgAHQAbwAgACcAcAByAHUAbgBpAG4AZwBzACcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAARQBGACAAcwBvAHUAcgBjAGUAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAHAAZQBjAGkAZgBpAGMAIAByAGUAZgBlAHIAZQBuAGMAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgA6ACAARgBvAG8AZAAgAHcAYQBzAHQAZQAsACAAZwByAGUAZQBuACAAdwBhAHMAdABlACwAIAB3AG8AbwBkACwAIABzAGwAdQBkAGcAZQAnACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgACcAQwBvAG0AcABvAHMAdABpAG4AZwA6ACAAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlACcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAJwBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAJwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyADoAIABWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAIAAoAHQALwBtADMAKQAgACgAVgBUAE0AdwApAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAVABNAHcAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAvAG0AMwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAxAC4AMgBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAyACwAIAAyACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAFYAVABNAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAuADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA5ADsAXABuACAAIAAgACAAIAAgACAAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA3ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgA0ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADYAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAOQBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEMAaABhAG4AZwBlAGQAIABjAG8AbAB1AG0AbgAgAGgAZQBhAGQAZQByACAAQwBGAHcAIAB0AG8AIABWAFQATQB3ACAAdABvACAAbQBhAHQAYwBoACAAdABpAHQAbABlACAAdgBhAHIAaQBhAGIAbABlAC4AXAAiACkAKQA7AFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAVQBuAGkAdABUAHkAcABlACwAXABuACAAIABTAFUATQBJAEYAUwAoAFwAbgAgACAAIAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALABcAG4AIAAgACAAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABcAG4AIAAgACAAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAVQBuAGkAdABUAHkAcABlAFwAbgAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdAAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16739,29 +16758,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
self-heal phantom Common_v03.xlsx external links in sync-xlf-to-excel-labs.ps1
Sync-CommonSheetsAcrossWorkbooks's sheet-copy step recreates the phantom
xl/externalLinks/* artifact (pointing at Common_v03.xlsx, no cached data, no
cell/name reference) on every workbook it touches - the cleanup from
yesterday didn't stick because the next build silently reintroduced it on
all 18 affected workbooks. Wire remove-phantom-external-links.ps1 -Commit
into the sync script itself, right after the Common-sheet propagation step,
so every build self-heals instead of needing a manual rerun. Verified: a
scoped sync run recreated the phantom link during its own Common-sheet-replace
step and the self-heal step removed it in the same run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v02.xlsx
+++ b/Excel/10_SolidWaste_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B007F79-B343-48ED-9198-78EB46E613FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD0FA77-3915-45C0-909D-5D4325777020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -19,11 +19,8 @@
     <sheet name="Input - Solid waste" sheetId="70" r:id="rId4"/>
     <sheet name="10.1.1-2 Solid waste treatment" sheetId="69" r:id="rId5"/>
     <sheet name="Constants - Solid Waste" sheetId="110" r:id="rId6"/>
-    <sheet name="Constants - Common" sheetId="128" r:id="rId7"/>
+    <sheet name="Constants - Common" sheetId="129" r:id="rId7"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId8"/>
-  </externalReferences>
   <definedNames>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -4550,26 +4547,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Home"/>
-      <sheetName val="Constants - Common"/>
-      <sheetName val="Acknowledgements"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -4657,16 +4634,16 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{2620DE19-BD98-481B-844A-8DE8AA67E6D6}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{13EC6376-0EDA-499E-BBAA-3B19EB568438}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
   <autoFilter ref="D36:E43" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{01C009EC-9C6B-49B4-A3AE-250C8CE8112F}" name="Gas">
+    <tableColumn id="1" xr3:uid="{C328050E-FB92-4C97-80F0-16560FDE6B1D}" name="Gas">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A3B74331-6B45-4D80-B7A7-5337AA87E03A}" name="CO2-e factor">
+    <tableColumn id="2" xr3:uid="{EAE55FFD-91C4-467B-B8FB-2A8E6E4A6327}" name="CO2-e factor">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4675,7 +4652,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{78F119C0-FF21-43AF-8686-044259BBC09C}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{2EADAD8B-9EEA-4579-B066-8C105E768D08}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
   <autoFilter ref="D47:H54" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4684,19 +4661,19 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{CCA9BFCA-5D5E-41A4-BB23-9521ABDCF323}" name="Gas">
+    <tableColumn id="1" xr3:uid="{C9934B05-DE9D-4497-A725-F3C9572C1784}" name="Gas">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{333051B1-81A7-4882-95F7-E8EA651054D1}" name="Conversion factor">
+    <tableColumn id="5" xr3:uid="{9BDA38AE-2016-4C11-933F-682BC1AE5D2A}" name="Conversion factor">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{86490AC6-6788-4809-9AE8-E4849393F9B6}" name="Conversion factor 1">
+    <tableColumn id="2" xr3:uid="{F5094EF0-BDB8-483B-B16B-B5B721C10CC9}" name="Conversion factor 1">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{1CAFD05C-FCC2-4D30-923F-6BA6207460FD}" name="Conversion factor 2">
+    <tableColumn id="3" xr3:uid="{7D45A8BF-2372-4462-842A-78176F3B1BF2}" name="Conversion factor 2">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{62D80E7C-7755-445A-BA58-C004CD5D0F2E}" name="Conversion factor combined">
+    <tableColumn id="4" xr3:uid="{DA570291-E2D2-4BA9-BAFA-1CB4FD805966}" name="Conversion factor combined">
       <calculatedColumnFormula>Table_GasToMolecularConversionFactor[[#This Row],[Conversion factor 1]]/Table_GasToMolecularConversionFactor[[#This Row],[Conversion factor 2]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4705,7 +4682,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{F36A2B59-4569-4B12-B867-DCA1C5ED1056}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{2FD9ADDB-3533-4A65-870C-5699C3EF683E}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
   <autoFilter ref="D89:S97" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4725,52 +4702,52 @@
     <filterColumn colId="15" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{27DFE9D9-2C4D-4602-B655-F050C31BAA61}" name="Climate zone" totalsRowCellStyle="Content bold">
+    <tableColumn id="1" xr3:uid="{EE0590A9-ED09-491E-AEC3-FCF242CB7376}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F19A45E4-25A1-4DE7-A9B6-4855B7FDF2E7}" name="MAT" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{BCCDCD9B-7481-4E2F-B896-4FB72A387FED}" name="MAT" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8E1D714D-45DE-4FBB-9975-41C68CE8B79A}" name="MAP" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{D2B2BDEE-B369-4444-B527-E893006B4FA0}" name="MAP" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{166C6EDF-61A9-47D5-935E-CCE44A776944}" name="Frost days per year" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{E732C349-18E6-4D9D-BA1C-FE8B59D7D15B}" name="Frost days per year" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{C715B81D-3778-42C9-9B91-0E800E220C70}" name="Elevation" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{303DF1C2-2350-4D45-AA36-ED38863763FE}" name="Elevation" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{29C04F46-59E8-4900-A14E-D7D36C2F0E62}" name="MAP:PET" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{FC51B0BB-F1DA-4262-B02A-D828303C9C76}" name="MAP:PET" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{34BC3595-15D2-4ED5-A837-708980C7733D}" name="Min temp" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{5E2F58A5-E01C-4DE1-9178-CA49B951DC2C}" name="Min temp" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{6E3DE317-C4A5-4729-AD91-315C8D959B53}" name="Max temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{C4B70C8A-E2B8-4845-8548-A9456B6722D0}" name="Max temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{F310B65E-0CBA-4DD4-B103-1F56E3990CCD}" name="Min rainfall" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{0CCF5866-BA37-4022-80F8-37662F9AB2EA}" name="Min rainfall" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{D0E7330C-BA59-4D74-B9D2-D9E7BCF660F2}" name="Max rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{73EDD18A-99EB-4E38-9D1E-337BCAE64070}" name="Max rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{76EF27D1-B984-4CFE-ADF3-08CF287F0A58}" name="Min frost days" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{30316D2A-4CAE-4455-8C3D-492D2DCBD053}" name="Min frost days" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{6E0A156C-EFB9-4B22-9ABF-0D1F8696B733}" name="Max frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{F82081DB-9EC8-4B20-95E2-62E270352400}" name="Max frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{6AE12849-873C-48E9-A4C5-6B8A50B3BCD5}" name="Min elevation" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{5B160519-4BA4-459D-B962-BFE522DFFB0D}" name="Min elevation" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{6B5888E7-7E27-4B37-9D3B-8DA24AE59C4F}" name="Max elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{86A1C9D0-D4DE-4668-8690-85A1670BD261}" name="Max elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{CD05F6D0-5B34-47C2-A227-5FC3E1AB9AE6}" name="Min MAP:PET" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{32494D7E-1C24-42BC-A598-85B9FF27B02D}" name="Min MAP:PET" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{FCCE3359-44AE-429E-82A1-8BC34DA17A0E}" name="Max MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{D1BF5C1A-E557-49F6-B044-B5111E6D80D0}" name="Max MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4779,16 +4756,16 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{1AEEE48A-E197-414C-94FF-88FD1833024D}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{9BACEC28-54F4-4D2B-A2D8-12CFBABEF176}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
   <autoFilter ref="D63:E77" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{6A2732CA-28B9-4CCD-B44E-97D64245ED12}" name="Climate zone" totalsRowCellStyle="Content bold">
+    <tableColumn id="1" xr3:uid="{2434BE68-48ED-4265-9E37-F2D27A95820A}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E4DEEEBC-476B-416E-A88C-126EAAF3D343}" name="Wet or Dry Zone" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{E4CDD59F-CBED-4486-AD4A-9D5CA0A6E0D7}" name="Wet or Dry Zone" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4797,7 +4774,7 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{E6BB6D0D-F94C-46A7-8DBF-6CC0807BC7CC}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{8B23EB57-2A24-46DB-ADCB-13266E08E100}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
   <autoFilter ref="D109:G112" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4805,16 +4782,16 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{29814AED-B44A-4393-A398-0C6BD7D8FD35}" name="Temperature Zone">
+    <tableColumn id="1" xr3:uid="{AB564272-7E43-46B0-BFD0-F572D7AA81E4}" name="Temperature Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8A52236C-5358-467B-A0D2-F1BB0BAEEF5B}" name="MAT">
+    <tableColumn id="2" xr3:uid="{74888402-0A3A-458C-9708-11D4E16A561B}" name="MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{61831EA1-76E4-47DF-ABC8-D21C4CE0F24C}" name="Min MAT">
+    <tableColumn id="3" xr3:uid="{30F2537C-9CD4-4C67-A5DF-E950ECD987F8}" name="Min MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DDBE3C16-3277-4229-A389-A85DB0C3927A}" name="Max MAT">
+    <tableColumn id="4" xr3:uid="{1CD1CFB0-19DC-481B-9116-61070A66297C}" name="Max MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4823,7 +4800,7 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{14916B19-CEF3-471B-86C8-5B8709CEDFF7}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{C4ED55DC-E783-402D-93C8-079F5B6C4975}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
   <autoFilter ref="D119:G121" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4831,16 +4808,16 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C2469925-09F2-46A7-B437-8D0C63B14845}" name="Rainfall Zone">
+    <tableColumn id="1" xr3:uid="{CC5F4695-99A9-4FA3-ACC5-E52DA281725B}" name="Rainfall Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E5EF70A6-5173-4048-9CF8-F4A49FA82CD8}" name="Annual rainfall">
+    <tableColumn id="2" xr3:uid="{B0915F74-FA66-427E-961D-1103F738271E}" name="Annual rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{ECEAF9F9-2992-4C76-8801-B60C107CF29B}" name="Min rainfall">
+    <tableColumn id="3" xr3:uid="{EF0DC8E0-0880-46C6-BD8C-21FB2019B7E8}" name="Min rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{893D1034-7B13-408A-BEA0-511C2BC3FD57}" name="Max rainfall">
+    <tableColumn id="4" xr3:uid="{503C2CFE-8277-4BF3-A67A-5949400BABC5}" name="Max rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4849,16 +4826,16 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{8BFDABF1-39EE-4F1A-A496-0A8F1F835C82}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{E5117961-FACC-4251-86C7-264B8FFFDAEC}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
   <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{9FDAFA40-FF9E-455E-9295-2D9A260BB1BC}" name="Leaching Zone">
+    <tableColumn id="1" xr3:uid="{499E70E9-BA3A-47D3-98DE-9DEB7862EC83}" name="Leaching Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B3D26D92-BF34-4003-A3EB-427770AB5BD4}" name="Leaching criteria">
+    <tableColumn id="2" xr3:uid="{CB2B961E-CA51-46E8-AD3A-8757B7D1CCD6}" name="Leaching criteria">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4867,16 +4844,16 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{1DAA5C12-62AE-4FC5-B846-EAFAECD7A654}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{EDF3F978-0171-40B1-B3DD-5CF1D3E18824}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
   <autoFilter ref="D153:E158" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{675D81EF-A676-4F1F-9BC4-743FBF5FDDC5}" name="Data source">
+    <tableColumn id="1" xr3:uid="{83D7A3DB-01E0-4C7D-A509-CDEC7B91442E}" name="Data source">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1CA89E49-C41F-4150-9368-12FC2D8B8E35}" name="Data score">
+    <tableColumn id="2" xr3:uid="{AFF8EB0A-41B7-4FDA-B015-6B46BA85121B}" name="Data score">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4885,16 +4862,16 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{5D1A3453-CFA5-49F0-9F50-0CA054FA2F74}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{E756EB14-7F8A-4AF9-89B6-4A619B1EA69E}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
   <autoFilter ref="D134:E136" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{5FDB0A66-3CCD-4216-AACF-68106D114098}" name="Is in leaching zone">
+    <tableColumn id="1" xr3:uid="{E18E07A4-4ACF-465A-B71D-64E61CFA7FB1}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A83B5834-C406-4353-B695-4AEA89ADCD15}" name="FracWET" dataDxfId="20">
+    <tableColumn id="2" xr3:uid="{C87CA644-108F-45EC-A29C-6DFD8D2BDD9F}" name="FracWET" dataDxfId="20">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4903,7 +4880,7 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{3FA240EF-7250-4ED5-A122-859FC209179A}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{ABBE80D6-B51C-4CDA-8275-8D54AA7A4DDC}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
   <autoFilter ref="D186:H199" xr:uid="{D41FBEA4-8379-4DF7-A068-BF94D364F1A2}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4912,19 +4889,19 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{6D803D77-65D8-4030-BDB8-0D50EF26FD06}" name="Production system j">
+    <tableColumn id="1" xr3:uid="{4B5D176C-19F4-4326-AB86-7C67C13FF3DA}" name="Production system j">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B21A730C-1310-4624-93C1-FC12D1B00DDB}" name="EFN2O">
+    <tableColumn id="2" xr3:uid="{F5ED76E6-B875-4CA5-9B21-9D023E73390A}" name="EFN2O">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{126C9A19-E20A-4DDC-A7ED-B210C0359266}" name="Production system only">
+    <tableColumn id="3" xr3:uid="{1B78CB92-719D-4874-9934-4FCE9BCE3475}" name="Production system only">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{F60F9E7D-83F5-476E-8270-FF6D44B67A4C}" name="Irrigation method">
+    <tableColumn id="4" xr3:uid="{F6E9DE14-9178-4B58-8AC8-3A9A4FF456C4}" name="Irrigation method">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A816AAE-81DE-4653-A60F-B4E8CF1C4E6A}" name="Rainfall zone">
+    <tableColumn id="5" xr3:uid="{AFEDFF0F-0FED-481A-8F39-4C6102CABB5A}" name="Rainfall zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4959,16 +4936,16 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="37" xr:uid="{7F1125FB-52D5-4751-BE93-D30710719CC3}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{BDE12DA4-B00E-4155-8309-3F58ADB005E9}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
   <autoFilter ref="D142:E147" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1C9FFCF4-4A29-4ABE-82BD-F3DACB8954C2}" name="Irrigation type i">
+    <tableColumn id="1" xr3:uid="{61CE0FFA-4CDD-4BA7-A452-E6668DD36FE0}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{86EE9F13-1AEA-4966-A7BF-6F0669A9C13A}" name="FracWET" dataDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{6F34C4D6-2644-4149-A432-7F2BC1F684BE}" name="FracWET" dataDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4977,16 +4954,16 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="38" xr:uid="{93627CD5-ED79-4088-9591-B09590CDF2A9}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{EE88CD00-1C0F-4D41-A840-CFB75BDC018E}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
   <autoFilter ref="D206:E208" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{04348CA0-C34B-42DF-80D1-DB94F5184729}" name="Climate zone">
+    <tableColumn id="1" xr3:uid="{A99775C0-483C-49FB-96F2-E8B7765FF2EE}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3068BB1E-C216-45F7-A1B2-3ED4B278BA8E}" name="EFPRP" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{92FD3274-10AF-4F4F-98F0-B68E3F04780E}" name="EFPRP" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4995,16 +4972,16 @@
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="39" xr:uid="{746C87DD-5686-488B-BA2D-4319EE4747A3}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{E6C8802C-BF04-425D-9C34-E56A86B54529}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
   <autoFilter ref="D212:E224" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{83A7B37F-2BDA-4414-86F7-3394268E0B73}" name="Month">
+    <tableColumn id="1" xr3:uid="{679D4915-5C33-4200-9E3D-145533AAF7C3}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D1F94E48-9EB5-421F-9182-287BD661FBBE}" name="Season" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{F7A60CCA-25DB-4DBB-B6C0-608B8495B287}" name="Season" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5013,7 +4990,7 @@
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="40" xr:uid="{8B0EAA03-144C-4774-A459-24C3F7ECD4C5}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{B8DD31D5-B3BA-4E7F-8B59-FD0C1F69A0E5}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
   <autoFilter ref="D231:S250" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5033,52 +5010,52 @@
     <filterColumn colId="15" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{BBB3E5AF-BEB8-437C-936A-F17811BF09CF}" name="Temperature zone">
+    <tableColumn id="1" xr3:uid="{21E1DFD8-4A18-41E8-B8F0-E7CB7F6FD5EC}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{204D7411-242F-4F7B-A700-C8688E43C368}" name="MAT (ºC)" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{71CB584D-4CD7-4B5F-8051-0D73E3756314}" name="MAT (ºC)" dataDxfId="16" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F7B19DCF-59FA-4318-93DD-3461DBE7644D}" name="Anaerobic lagoon" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{B8946676-EE29-4950-B84F-3BC2D82AFC14}" name="Anaerobic lagoon" dataDxfId="15" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8009790C-A1CA-435F-9146-7B7EDE0F60A4}" name="Digester / covered lagoons" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{15B31438-0CB8-4D4B-8DB8-371A74F7579E}" name="Digester / covered lagoons" dataDxfId="14" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{AE4C5198-CE55-41E2-ACF1-681E6050F2D4}" name="Liquid systems" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{ED478E11-2B9A-409F-8E13-24D702F393B5}" name="Liquid systems" dataDxfId="13" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{AA77C933-1912-4073-AF6E-3716241883B9}" name="Daily spread" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{753D73B3-329E-4CA4-8892-D317AC5DEF99}" name="Daily spread" dataDxfId="12" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{106A7FA1-5FF4-4723-94F4-3E9E7CBF1250}" name="Composting (passive windrow)" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{4D148273-2490-46F0-83EC-F28B2EBAE4DA}" name="Composting (passive windrow)" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4669A826-8AF7-4E7D-9AE7-B35DB6260008}" name="Solid storage" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{DE378BC6-60D7-4699-805C-D9AC1B15231B}" name="Solid storage" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{4999EA1C-9103-4061-AC89-73C9872D435C}" name="Pit storage" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{BC0863DC-DAB7-40BE-8911-E9A9DFD63EEE}" name="Pit storage" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{2BC94F92-2320-41DA-8691-E93B9D33B2B4}" name="Deep litter" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{AB969467-0898-4067-8474-90814E64B994}" name="Deep litter" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{99939850-BBB8-440E-9EE3-A9CA06EBE993}" name="Poultry manure with bedding" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{BFD1EE98-B0C8-4D9C-BE89-1BF44D3DA366}" name="Poultry manure with bedding" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{567E6EDF-41A4-40FF-A6A0-FA26B71CB44B}" name="Poultry manure without bedding" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{4B6D9474-35E0-4C3C-99D2-9F50DD4CDF49}" name="Poultry manure without bedding" dataDxfId="6" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{0E5A08A9-2155-472F-95A6-4009F869E785}" name="Direct processing" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{DE4D7369-BB2D-43AA-8F50-628A73F5CB8B}" name="Direct processing" dataDxfId="5" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{0A53E068-6009-4BB8-8B7D-A522161F6009}" name="Direct application" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{C4ABB577-EC03-4E4B-B87C-7F5F74B6356D}" name="Direct application" dataDxfId="4" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{5D5FB4D9-FF92-4150-92DA-04A9935F2819}" name="Pasture range and paddock" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{D623DAF3-D70F-4B5B-9D72-36A961F94E1E}" name="Pasture range and paddock" dataDxfId="3" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{35F85007-82F1-4A96-86FF-876DA0061D75}" name="MAT raw" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{0825DE9E-7EFD-4132-B182-D37A723AF24D}" name="MAT raw" dataDxfId="2" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5087,16 +5064,16 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="41" xr:uid="{1321004A-E71E-4324-8584-E52D09319395}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{27A5FDBF-EB52-431E-9F01-1F9C07DBBDD4}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
   <autoFilter ref="D257:E259" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D6F2F64E-9B4D-4847-A34E-10B559D9C9F6}" name="Climate Zone">
+    <tableColumn id="1" xr3:uid="{CA1FB309-72EF-4ECE-9117-475B3F8B29B3}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{5AA32039-8F3E-4678-8CD5-7C4A1ABB9B63}" name="EFNi &amp; EFN2Oi" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{8D03B58D-6148-414D-974D-21D167EB202A}" name="EFNi &amp; EFN2Oi" dataDxfId="1" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5105,64 +5082,64 @@
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="42" xr:uid="{7809F716-2A2A-47FA-B7B7-4737229AC065}" name="Table_SourceData_DataQuality_TemporalRepresentativeness" displayName="Table_SourceData_DataQuality_TemporalRepresentativeness" ref="D265:F270" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="46" xr:uid="{A72C1C18-5D46-49DA-8F7F-51B8B9D2920C}" name="Table_SourceData_DataQuality_TemporalRepresentativeness" displayName="Table_SourceData_DataQuality_TemporalRepresentativeness" ref="D265:F270" totalsRowShown="0">
   <autoFilter ref="D265:F270" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{2C9063BD-C39C-4614-9F12-7C498F509602}" name="Description" dataDxfId="0" dataCellStyle="Content normal"/>
-    <tableColumn id="1" xr3:uid="{AB695E03-6FE6-4560-BD9A-CD6FB74A4841}" name="ID"/>
-    <tableColumn id="3" xr3:uid="{5A4FE66A-2A87-4FA4-B114-81F483B73EB3}" name="Score"/>
+    <tableColumn id="2" xr3:uid="{A382F094-D822-4061-A637-32327308BEEC}" name="Description" dataDxfId="0" dataCellStyle="Content normal"/>
+    <tableColumn id="1" xr3:uid="{2E6D07F2-30C8-4E24-8AE2-FB99C88B4C43}" name="ID"/>
+    <tableColumn id="3" xr3:uid="{8A2B12E3-C908-459E-9D86-86B5EDB7A47C}" name="Score"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="43" xr:uid="{14724696-D7A8-4C6E-9B11-538CB153555D}" name="Table_SourceData_DataQuality_SpatialRepresentativeness" displayName="Table_SourceData_DataQuality_SpatialRepresentativeness" ref="D274:F279" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="47" xr:uid="{EFCF913B-4CDB-48CD-97ED-32542E115687}" name="Table_SourceData_DataQuality_SpatialRepresentativeness" displayName="Table_SourceData_DataQuality_SpatialRepresentativeness" ref="D274:F279" totalsRowShown="0">
   <autoFilter ref="D274:F279" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{3553CCAF-8A29-4080-8F21-B15ED6FEFDE1}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{384F1974-F0E3-44F2-8B01-C3E7C2019A2E}" name="ID"/>
-    <tableColumn id="3" xr3:uid="{8C8A74B4-2466-4E4D-BB89-FD4620317D14}" name="Score"/>
+    <tableColumn id="1" xr3:uid="{B099C4F5-451A-4798-A3C3-C67352C82818}" name="Description"/>
+    <tableColumn id="2" xr3:uid="{6ADD1DE9-1E2E-4C67-A7F5-311F74D67BE2}" name="ID"/>
+    <tableColumn id="3" xr3:uid="{FEB599D0-7E37-4D3C-B483-6EDEEDA6B652}" name="Score"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="44" xr:uid="{F3FC9567-161F-4238-8F4A-5ECB030F1D68}" name="Table_SourceData_DataQuality_SampleSize" displayName="Table_SourceData_DataQuality_SampleSize" ref="D283:F288" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="48" xr:uid="{74AE3B2E-93F0-4F07-B1DF-B6ED6F2EB69C}" name="Table_SourceData_DataQuality_SampleSize" displayName="Table_SourceData_DataQuality_SampleSize" ref="D283:F288" totalsRowShown="0">
   <autoFilter ref="D283:F288" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{4AC60456-C435-4920-9F3E-933EC33C1ACD}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{1AF54846-4887-41CC-9E9E-55EA91E2F7B0}" name="ID"/>
-    <tableColumn id="3" xr3:uid="{A5D00AC9-0D1E-474B-9C8F-22AE7DA0DB01}" name="Score"/>
+    <tableColumn id="1" xr3:uid="{307213C5-6777-4215-8824-C259E2CE121E}" name="Description"/>
+    <tableColumn id="2" xr3:uid="{FA718452-8CB8-40F0-8D47-1965C69073F9}" name="ID"/>
+    <tableColumn id="3" xr3:uid="{07F432A1-4208-49C7-9954-B8B182FF628F}" name="Score"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="45" xr:uid="{9F431637-E8F0-44E5-9AF4-528A066538BC}" name="Table_SourceData_DataQuality_Scope3" displayName="Table_SourceData_DataQuality_Scope3" ref="D292:F297" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="49" xr:uid="{7677EBCC-56FB-4DE5-BFBE-988369801BEA}" name="Table_SourceData_DataQuality_Scope3" displayName="Table_SourceData_DataQuality_Scope3" ref="D292:F297" totalsRowShown="0">
   <autoFilter ref="D292:F297" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{6A398FBC-C5B4-476A-8F3E-AC21BEF54585}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{DFFB7A20-6DCD-48D0-87E7-FD356F55DBA1}" name="ID"/>
-    <tableColumn id="3" xr3:uid="{96FCBA22-F077-40C3-AE14-7A21817FC90D}" name="Score"/>
+    <tableColumn id="1" xr3:uid="{2AB0A2E9-8E35-4591-B8A4-FA98C906E8EB}" name="Description"/>
+    <tableColumn id="2" xr3:uid="{22AA4894-98D6-4EC7-B095-A46C0B32F460}" name="ID"/>
+    <tableColumn id="3" xr3:uid="{D694B58D-0AB0-4946-8648-70ADB2FD0A9C}" name="Score"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5243,20 +5220,20 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6EABCA6F-C222-4895-A37A-C20DF9DEFFEC}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C12DB254-862F-4810-97E9-D3B961DE7BC5}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
   <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B2007ADB-B76B-4D97-B60C-258785E6E15F}" name="State/Territory">
+    <tableColumn id="1" xr3:uid="{3627AF9A-5057-427B-A601-42D57044EF7C}" name="State/Territory">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{73B353BF-4543-4131-8839-E8D248923F46}" name="Common Name">
+    <tableColumn id="2" xr3:uid="{FCF3211B-8822-4BDD-A557-189A557282A9}" name="Common Name">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{378480C6-E579-43EB-8A39-00B86FA50B83}" name="Abbreviation">
+    <tableColumn id="3" xr3:uid="{0CD29EA2-AA75-4A0A-8378-94A46EE4AA24}" name="Abbreviation">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5265,12 +5242,12 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{3E47D686-04FE-4C61-9126-799AFC028C0E}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E8C3BCAE-A949-4888-B1D3-F98AE74CA0A1}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
   <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{2F0F0A2E-E2AA-4831-AFA8-654F2684B2E3}" name="SA 4 Name">
+    <tableColumn id="1" xr3:uid="{867D7E20-10F8-4B61-8561-C76DAE03D25B}" name="SA 4 Name">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -12598,7 +12575,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855DD939-2360-45F2-BA7B-4DEEA3DC75A7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51E3E444-BBEF-45FC-817E-D43176765775}">
   <sheetPr>
     <tabColor theme="2" tint="-0.499984740745262"/>
   </sheetPr>
@@ -17038,14 +17015,7 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA0ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxADoAIABXAGEAcwB0AGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AbABpAGQAIABXAGEAcwB0AGUAIABUAHIAZQBhAHQAbQBlAG4AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXABuAEUAXwBnAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAGcAPQBcAFwAcwB1AG0AXwB0AFwAXABzAHUAbQBfAHcAKABRAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB3AHQAZwApAFwAbgBRAF8AdwB0ACAAPQAgAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAIAAoAHQAKQBcAG4ARQBGAF8AdwB0AGcAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAdAAgAEMATwAyAGUALwB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AdwB0ACwAIABFAEYAXwB3AHQAZwAsAFwAbgAgACAAIAAgAFEAXwB3AHQAIAAqACAARQBGAF8AdwB0AGcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdABcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHcAKABRAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewB3AHQAZwB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzAFwAIgAsACAAXAAiAHQAXAAiACwAIABcACIAUwB1AG0AIABvAGYAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAHcAdABnAFwAIgAsACAAXAAiAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAdAAgAEMATwAyAGUALwB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGcAXAAiACwAIABcACIAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHYAbwBsAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAdgBvAGwAdQBtAGUAIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAdABvAG4AbgBlAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAxADAALgAxAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAG0AYQBzAHMAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AYQBzAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAIAB2AGEAcgBpAGEAYgBsAGUAcwAgAHQAbwAgAGMAbABlAGEAcgBsAHkAIAB0AHIAYQBjAGsAIABpAG4AcAB1AHQAIABvAHIAIABjAGEAbABjAHUAbABhAHQAZQBkACAAUQAgAHYAYQBsAHUAZQBzAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXABuAFEAXwB3AHQAXABuAHQAXABuAFEAXwB3AHQAPQBWAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXABuAFYAXwB3AHQAIAA9ACAAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAG0AMwApAFwAbgBWAFQATQBfAHcAIAA9ACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgACgAdAAvAG0AMwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAXwB3AHQALAAgAFYAVABNAF8AdwAsAFwAbgAgACAAIAAgAFYAXwB3AHQAIAAqACAAVgBUAE0AXwB3AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AdwB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB7AHcAdAB9AD0AVgBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBfAHcAdABcACIALAAgAFwAIgB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgBtADMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFQATQBfAHcAXAAiACwAIABcACIAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgB0AC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBGAHcAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAgAEMATwAyAGUAIAAvACAAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADEAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzADUALAAgADQALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIAB0AHkAcABlACAAdABcACIALAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBFAEYAdwB0AFwAIgAsACAAXAAiAEUARgAgAHMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAyAC4AMQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4ANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAyAC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA0ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUALAAgAGcAcgBlAGUAbgAgAHcAYQBzAHQAZQAsACAAdwBvAG8AZAAsACAAcwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMQA2ADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMwA2ADYANwAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADQAOQAxADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgAxADEAMAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA1ADMANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgA0ADkALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABcAHUAMAAwADIANwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZABcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AHAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAB1ADAAMAAyADcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAFwAdQAwADAAMgA3AHAAcgB1AG4AbgBpAG4AZwBzAFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcAcAByAHUAbgBpAG4AZwBzAFwAdQAwADAAMgA3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAEUARgAgAHMAbwB1AHIAYwBlACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBwAGUAYwBpAGYAaQBjACAAcgBlAGYAZQByAGUAbgBjAGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgAFwAdQAwADAAMgA3AEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuADoAIABGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAdQAwADAAMgA3ACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgAFwAdQAwADAAMgA3AEMAbwBtAHAAbwBzAHQAaQBuAGcAOgAgAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcAHUAMAAwADIANwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAB1ADAAMAAyADcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AVABhAGIAbABlACAAQQAuADQALgAxAC4AMgA6ACAAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzACAAKAB0AC8AbQAzACkAIAAoAFYAVABNAHcAKQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAFQATQB3AFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQALwBtADMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMgAsACAAMgAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBWAFQATQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgA1ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMgA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBvAG8AZABcACIALAAgADAALgAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4ANwAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgB1AGIAYgBlAHIAIABhAG4AZAAgAGwAZQBhAHQAaABlAHIAXAAiACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwAC4ANAAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA2ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbgBzAHQAcgB1AGMAdABpAG8AbgAgAGEAbgBkACAAZABlAG0AbwBsAGkAdABpAG8AbgAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADkAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABDAGgAYQBuAGcAZQBkACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgAgAEMARgB3ACAAdABvACAAVgBUAE0AdwAgAHQAbwAgAG0AYQB0AGMAaAAgAHQAaQB0AGwAZQAgAHYAYQByAGkAYQBiAGwAZQAuAFwAIgApACkAOwBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABUAHkAcABlACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFUAbgBpAHQAVAB5AHAAZQAsAFwAbgAgACAAUwBVAE0ASQBGAFMAKABcAG4AIAAgACAAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgACAAVAByAGUAYQB0AG0AZQBuAHQAQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABUAHkAcABlACwAXABuACAAIAAgACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVwBhAHMAdABlAFQAeQBwAGUALABcAG4AIAAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAXABuACAAIAAgACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAFUAbgBpAHQAVAB5AHAAZQBcAG4AIAAgACkAXABuACkAOwAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17058,7 +17028,14 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA0ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxADoAIABXAGEAcwB0AGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AbABpAGQAIABXAGEAcwB0AGUAIABUAHIAZQBhAHQAbQBlAG4AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXABuAEUAXwBnAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAGcAPQBcAFwAcwB1AG0AXwB0AFwAXABzAHUAbQBfAHcAKABRAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB3AHQAZwApAFwAbgBRAF8AdwB0ACAAPQAgAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAIAAoAHQAKQBcAG4ARQBGAF8AdwB0AGcAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAdAAgAEMATwAyAGUALwB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AdwB0ACwAIABFAEYAXwB3AHQAZwAsAFwAbgAgACAAIAAgAFEAXwB3AHQAIAAqACAARQBGAF8AdwB0AGcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdABcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHcAKABRAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewB3AHQAZwB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzAFwAIgAsACAAXAAiAHQAXAAiACwAIABcACIAUwB1AG0AIABvAGYAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAHcAdABnAFwAIgAsACAAXAAiAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAdAAgAEMATwAyAGUALwB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGcAXAAiACwAIABcACIAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHYAbwBsAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAdgBvAGwAdQBtAGUAIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAdABvAG4AbgBlAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAxADAALgAxAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAG0AYQBzAHMAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AYQBzAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAIAB2AGEAcgBpAGEAYgBsAGUAcwAgAHQAbwAgAGMAbABlAGEAcgBsAHkAIAB0AHIAYQBjAGsAIABpAG4AcAB1AHQAIABvAHIAIABjAGEAbABjAHUAbABhAHQAZQBkACAAUQAgAHYAYQBsAHUAZQBzAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXABuAFEAXwB3AHQAXABuAHQAXABuAFEAXwB3AHQAPQBWAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXABuAFYAXwB3AHQAIAA9ACAAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAG0AMwApAFwAbgBWAFQATQBfAHcAIAA9ACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgACgAdAAvAG0AMwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAXwB3AHQALAAgAFYAVABNAF8AdwAsAFwAbgAgACAAIAAgAFYAXwB3AHQAIAAqACAAVgBUAE0AXwB3AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AdwB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB7AHcAdAB9AD0AVgBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBfAHcAdABcACIALAAgAFwAIgB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgBtADMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFQATQBfAHcAXAAiACwAIABcACIAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgB0AC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBGAHcAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAgAEMATwAyAGUAIAAvACAAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADEAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzADUALAAgADQALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIAB0AHkAcABlACAAdABcACIALAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBFAEYAdwB0AFwAIgAsACAAXAAiAEUARgAgAHMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAyAC4AMQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4ANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAyAC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA0ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUALAAgAGcAcgBlAGUAbgAgAHcAYQBzAHQAZQAsACAAdwBvAG8AZAAsACAAcwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMQA2ADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMwA2ADYANwAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADQAOQAxADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgAxADEAMAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA1ADMANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgA0ADkALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABcAHUAMAAwADIANwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZABcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AHAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAB1ADAAMAAyADcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAFwAdQAwADAAMgA3AHAAcgB1AG4AbgBpAG4AZwBzAFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcAcAByAHUAbgBpAG4AZwBzAFwAdQAwADAAMgA3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAEUARgAgAHMAbwB1AHIAYwBlACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBwAGUAYwBpAGYAaQBjACAAcgBlAGYAZQByAGUAbgBjAGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgAFwAdQAwADAAMgA3AEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuADoAIABGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAdQAwADAAMgA3ACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgAFwAdQAwADAAMgA3AEMAbwBtAHAAbwBzAHQAaQBuAGcAOgAgAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcAHUAMAAwADIANwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAB1ADAAMAAyADcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AVABhAGIAbABlACAAQQAuADQALgAxAC4AMgA6ACAAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzACAAKAB0AC8AbQAzACkAIAAoAFYAVABNAHcAKQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAFQATQB3AFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQALwBtADMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMgAsACAAMgAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBWAFQATQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgA1ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMgA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBvAG8AZABcACIALAAgADAALgAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4ANwAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgB1AGIAYgBlAHIAIABhAG4AZAAgAGwAZQBhAHQAaABlAHIAXAAiACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwAC4ANAAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA2ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbgBzAHQAcgB1AGMAdABpAG8AbgAgAGEAbgBkACAAZABlAG0AbwBsAGkAdABpAG8AbgAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADkAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABDAGgAYQBuAGcAZQBkACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgAgAEMARgB3ACAAdABvACAAVgBUAE0AdwAgAHQAbwAgAG0AYQB0AGMAaAAgAHQAaQB0AGwAZQAgAHYAYQByAGkAYQBiAGwAZQAuAFwAIgApACkAOwBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABUAHkAcABlACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFUAbgBpAHQAVAB5AHAAZQAsAFwAbgAgACAAUwBVAE0ASQBGAFMAKABcAG4AIAAgACAAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgACAAVAByAGUAYQB0AG0AZQBuAHQAQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABUAHkAcABlACwAXABuACAAIAAgACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVwBhAHMAdABlAFQAeQBwAGUALABcAG4AIAAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAXABuACAAIAAgACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAFUAbgBpAHQAVAB5AHAAZQBcAG4AIAAgACkAXABuACkAOwAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17257,12 +17234,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17276,9 +17250,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
misc scope 3 excel updates
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v02.xlsx
+++ b/Excel/10_SolidWaste_WIP_v02.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD0FA77-3915-45C0-909D-5D4325777020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F51DF0-C84C-424D-9819-34B9E4671CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="37170" windowHeight="19920" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -2235,6 +2235,358 @@
   <dxfs count="75">
     <dxf>
       <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -3123,358 +3475,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <family val="2"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -4109,10 +4109,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -4325,10 +4322,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -4705,49 +4699,49 @@
     <tableColumn id="1" xr3:uid="{EE0590A9-ED09-491E-AEC3-FCF242CB7376}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{BCCDCD9B-7481-4E2F-B896-4FB72A387FED}" name="MAT" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{BCCDCD9B-7481-4E2F-B896-4FB72A387FED}" name="MAT" totalsRowDxfId="62" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{D2B2BDEE-B369-4444-B527-E893006B4FA0}" name="MAP" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{D2B2BDEE-B369-4444-B527-E893006B4FA0}" name="MAP" totalsRowDxfId="61" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{E732C349-18E6-4D9D-BA1C-FE8B59D7D15B}" name="Frost days per year" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{E732C349-18E6-4D9D-BA1C-FE8B59D7D15B}" name="Frost days per year" totalsRowDxfId="60" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{303DF1C2-2350-4D45-AA36-ED38863763FE}" name="Elevation" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{303DF1C2-2350-4D45-AA36-ED38863763FE}" name="Elevation" totalsRowDxfId="59" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{FC51B0BB-F1DA-4262-B02A-D828303C9C76}" name="MAP:PET" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{FC51B0BB-F1DA-4262-B02A-D828303C9C76}" name="MAP:PET" totalsRowDxfId="58" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{5E2F58A5-E01C-4DE1-9178-CA49B951DC2C}" name="Min temp" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{5E2F58A5-E01C-4DE1-9178-CA49B951DC2C}" name="Min temp" totalsRowDxfId="57" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{C4B70C8A-E2B8-4845-8548-A9456B6722D0}" name="Max temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{C4B70C8A-E2B8-4845-8548-A9456B6722D0}" name="Max temp" totalsRowDxfId="56" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{0CCF5866-BA37-4022-80F8-37662F9AB2EA}" name="Min rainfall" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{0CCF5866-BA37-4022-80F8-37662F9AB2EA}" name="Min rainfall" totalsRowDxfId="55" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{73EDD18A-99EB-4E38-9D1E-337BCAE64070}" name="Max rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{73EDD18A-99EB-4E38-9D1E-337BCAE64070}" name="Max rainfall" totalsRowDxfId="54" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{30316D2A-4CAE-4455-8C3D-492D2DCBD053}" name="Min frost days" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{30316D2A-4CAE-4455-8C3D-492D2DCBD053}" name="Min frost days" totalsRowDxfId="53" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{F82081DB-9EC8-4B20-95E2-62E270352400}" name="Max frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{F82081DB-9EC8-4B20-95E2-62E270352400}" name="Max frost days" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{5B160519-4BA4-459D-B962-BFE522DFFB0D}" name="Min elevation" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{5B160519-4BA4-459D-B962-BFE522DFFB0D}" name="Min elevation" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{86A1C9D0-D4DE-4668-8690-85A1670BD261}" name="Max elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{86A1C9D0-D4DE-4668-8690-85A1670BD261}" name="Max elevation" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{32494D7E-1C24-42BC-A598-85B9FF27B02D}" name="Min MAP:PET" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{32494D7E-1C24-42BC-A598-85B9FF27B02D}" name="Min MAP:PET" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{D1BF5C1A-E557-49F6-B044-B5111E6D80D0}" name="Max MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{D1BF5C1A-E557-49F6-B044-B5111E6D80D0}" name="Max MAP:PET" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4765,7 +4759,7 @@
     <tableColumn id="1" xr3:uid="{2434BE68-48ED-4265-9E37-F2D27A95820A}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E4CDD59F-CBED-4486-AD4A-9D5CA0A6E0D7}" name="Wet or Dry Zone" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{E4CDD59F-CBED-4486-AD4A-9D5CA0A6E0D7}" name="Wet or Dry Zone" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4871,7 +4865,7 @@
     <tableColumn id="1" xr3:uid="{E18E07A4-4ACF-465A-B71D-64E61CFA7FB1}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C87CA644-108F-45EC-A29C-6DFD8D2BDD9F}" name="FracWET" dataDxfId="20">
+    <tableColumn id="2" xr3:uid="{C87CA644-108F-45EC-A29C-6DFD8D2BDD9F}" name="FracWET" dataDxfId="46">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4921,13 +4915,13 @@
     <tableColumn id="1" xr3:uid="{27ECD0A0-9936-4A60-BCC5-02F0C62FDA6C}" name="Treatment type t">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B7AF1F5E-7BAC-4FF7-B59E-F905655514F2}" name="Waste type w" dataDxfId="62" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B7AF1F5E-7BAC-4FF7-B59E-F905655514F2}" name="Waste type w" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{EEC6B364-DA50-41AA-A530-330FAEE98233}" name="EFwt" dataDxfId="61" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{EEC6B364-DA50-41AA-A530-330FAEE98233}" name="EFwt" dataDxfId="24" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{01FD94D2-85D3-4478-AB5E-04E4027C2978}" name="EF source" dataDxfId="60" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{01FD94D2-85D3-4478-AB5E-04E4027C2978}" name="EF source" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4945,7 +4939,7 @@
     <tableColumn id="1" xr3:uid="{61CE0FFA-4CDD-4BA7-A452-E6668DD36FE0}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6F34C4D6-2644-4149-A432-7F2BC1F684BE}" name="FracWET" dataDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{6F34C4D6-2644-4149-A432-7F2BC1F684BE}" name="FracWET" dataDxfId="45" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4963,7 +4957,7 @@
     <tableColumn id="1" xr3:uid="{A99775C0-483C-49FB-96F2-E8B7765FF2EE}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{92FD3274-10AF-4F4F-98F0-B68E3F04780E}" name="EFPRP" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{92FD3274-10AF-4F4F-98F0-B68E3F04780E}" name="EFPRP" dataDxfId="44" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4981,7 +4975,7 @@
     <tableColumn id="1" xr3:uid="{679D4915-5C33-4200-9E3D-145533AAF7C3}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F7A60CCA-25DB-4DBB-B6C0-608B8495B287}" name="Season" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{F7A60CCA-25DB-4DBB-B6C0-608B8495B287}" name="Season" dataDxfId="43" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5013,49 +5007,49 @@
     <tableColumn id="1" xr3:uid="{21E1DFD8-4A18-41E8-B8F0-E7CB7F6FD5EC}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{71CB584D-4CD7-4B5F-8051-0D73E3756314}" name="MAT (ºC)" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{71CB584D-4CD7-4B5F-8051-0D73E3756314}" name="MAT (ºC)" dataDxfId="42" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B8946676-EE29-4950-B84F-3BC2D82AFC14}" name="Anaerobic lagoon" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{B8946676-EE29-4950-B84F-3BC2D82AFC14}" name="Anaerobic lagoon" dataDxfId="41" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{15B31438-0CB8-4D4B-8DB8-371A74F7579E}" name="Digester / covered lagoons" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{15B31438-0CB8-4D4B-8DB8-371A74F7579E}" name="Digester / covered lagoons" dataDxfId="40" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{ED478E11-2B9A-409F-8E13-24D702F393B5}" name="Liquid systems" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{ED478E11-2B9A-409F-8E13-24D702F393B5}" name="Liquid systems" dataDxfId="39" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{753D73B3-329E-4CA4-8892-D317AC5DEF99}" name="Daily spread" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{753D73B3-329E-4CA4-8892-D317AC5DEF99}" name="Daily spread" dataDxfId="38" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{4D148273-2490-46F0-83EC-F28B2EBAE4DA}" name="Composting (passive windrow)" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{4D148273-2490-46F0-83EC-F28B2EBAE4DA}" name="Composting (passive windrow)" dataDxfId="37" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{DE378BC6-60D7-4699-805C-D9AC1B15231B}" name="Solid storage" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{DE378BC6-60D7-4699-805C-D9AC1B15231B}" name="Solid storage" dataDxfId="36" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{BC0863DC-DAB7-40BE-8911-E9A9DFD63EEE}" name="Pit storage" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{BC0863DC-DAB7-40BE-8911-E9A9DFD63EEE}" name="Pit storage" dataDxfId="35" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{AB969467-0898-4067-8474-90814E64B994}" name="Deep litter" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{AB969467-0898-4067-8474-90814E64B994}" name="Deep litter" dataDxfId="34" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BFD1EE98-B0C8-4D9C-BE89-1BF44D3DA366}" name="Poultry manure with bedding" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{BFD1EE98-B0C8-4D9C-BE89-1BF44D3DA366}" name="Poultry manure with bedding" dataDxfId="33" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4B6D9474-35E0-4C3C-99D2-9F50DD4CDF49}" name="Poultry manure without bedding" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{4B6D9474-35E0-4C3C-99D2-9F50DD4CDF49}" name="Poultry manure without bedding" dataDxfId="32" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DE4D7369-BB2D-43AA-8F50-628A73F5CB8B}" name="Direct processing" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{DE4D7369-BB2D-43AA-8F50-628A73F5CB8B}" name="Direct processing" dataDxfId="31" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{C4ABB577-EC03-4E4B-B87C-7F5F74B6356D}" name="Direct application" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{C4ABB577-EC03-4E4B-B87C-7F5F74B6356D}" name="Direct application" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{D623DAF3-D70F-4B5B-9D72-36A961F94E1E}" name="Pasture range and paddock" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{D623DAF3-D70F-4B5B-9D72-36A961F94E1E}" name="Pasture range and paddock" dataDxfId="29" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{0825DE9E-7EFD-4132-B182-D37A723AF24D}" name="MAT raw" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{0825DE9E-7EFD-4132-B182-D37A723AF24D}" name="MAT raw" dataDxfId="28" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5073,7 +5067,7 @@
     <tableColumn id="1" xr3:uid="{CA1FB309-72EF-4ECE-9117-475B3F8B29B3}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8D03B58D-6148-414D-974D-21D167EB202A}" name="EFNi &amp; EFN2Oi" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{8D03B58D-6148-414D-974D-21D167EB202A}" name="EFNi &amp; EFN2Oi" dataDxfId="27" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5089,7 +5083,7 @@
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{A382F094-D822-4061-A637-32327308BEEC}" name="Description" dataDxfId="0" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{A382F094-D822-4061-A637-32327308BEEC}" name="Description" dataDxfId="26" dataCellStyle="Content normal"/>
     <tableColumn id="1" xr3:uid="{2E6D07F2-30C8-4E24-8AE2-FB99C88B4C43}" name="ID"/>
     <tableColumn id="3" xr3:uid="{8A2B12E3-C908-459E-9D86-86B5EDB7A47C}" name="Score"/>
   </tableColumns>
@@ -5155,7 +5149,7 @@
     <tableColumn id="1" xr3:uid="{E899A810-DA34-4DD3-9420-7017118A50BC}" name="Waste type w">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data(), Table_SourceData_WasteSolid_VolumeToMassConversion[[#Headers],[Waste type w]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EC8E9200-43B6-459C-B7A6-907C4A1A3CDE}" name="VTMw" dataDxfId="59" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{EC8E9200-43B6-459C-B7A6-907C4A1A3CDE}" name="VTMw" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data(), Table_SourceData_WasteSolid_VolumeToMassConversion[[#Headers],[Waste type w]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5178,7 +5172,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}" name="Table_WasteTypes_Incineration" displayName="Table_WasteTypes_Incineration" ref="K16:K26" totalsRowShown="0" headerRowDxfId="58" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}" name="Table_WasteTypes_Incineration" displayName="Table_WasteTypes_Incineration" ref="K16:K26" totalsRowShown="0" headerRowDxfId="21" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="K16:K26" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
@@ -5192,12 +5186,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}" name="Table_WasteTypes_Composting" displayName="Table_WasteTypes_Composting" ref="M16:M21" totalsRowShown="0" headerRowDxfId="57" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}" name="Table_WasteTypes_Composting" displayName="Table_WasteTypes_Composting" ref="M16:M21" totalsRowShown="0" headerRowDxfId="20" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="M16:M21" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{5B9ABACD-52AE-4D64-BCA6-1DA86A1A3FC3}" name="Waste type w" totalsRowDxfId="56" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{5B9ABACD-52AE-4D64-BCA6-1DA86A1A3FC3}" name="Waste type w" totalsRowDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula>E40</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5206,12 +5200,12 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}" name="Table_WasteTypes_Anaerobicdigestion" displayName="Table_WasteTypes_Anaerobicdigestion" ref="O16:O21" totalsRowShown="0" headerRowDxfId="55" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}" name="Table_WasteTypes_Anaerobicdigestion" displayName="Table_WasteTypes_Anaerobicdigestion" ref="O16:O21" totalsRowShown="0" headerRowDxfId="18" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="O16:O21" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{2D7DB5DA-05BB-4621-B5A8-576415999BBC}" name="Waste type w" totalsRowDxfId="54" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{2D7DB5DA-05BB-4621-B5A8-576415999BBC}" name="Waste type w" totalsRowDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula>E46</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7300,87 +7294,87 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F162:F163">
-    <cfRule type="cellIs" dxfId="53" priority="20" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="20" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F174:F175">
-    <cfRule type="cellIs" dxfId="52" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="15" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F186:F187">
-    <cfRule type="cellIs" dxfId="51" priority="18" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="18" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F274:F275">
-    <cfRule type="cellIs" dxfId="50" priority="93" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="93" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F279:F280">
-    <cfRule type="cellIs" dxfId="49" priority="92" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="92" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F284:F285">
-    <cfRule type="cellIs" dxfId="48" priority="91" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="91" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F308:F309">
-    <cfRule type="cellIs" dxfId="47" priority="85" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="85" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F313:F314">
-    <cfRule type="cellIs" dxfId="46" priority="84" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="84" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F318:F319">
-    <cfRule type="cellIs" dxfId="45" priority="83" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="83" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I33 F71">
-    <cfRule type="cellIs" dxfId="44" priority="62" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="62" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I79:I83">
-    <cfRule type="cellIs" dxfId="43" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I87 I146">
-    <cfRule type="cellIs" dxfId="42" priority="74" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="74" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I98:I100">
-    <cfRule type="cellIs" dxfId="41" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I104:I107">
-    <cfRule type="cellIs" dxfId="40" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I111:I115">
-    <cfRule type="cellIs" dxfId="39" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J8 I65:I66 H67:H69 I68 I70:I72 I74:I75 I226 I232 E234:G234">
-    <cfRule type="cellIs" dxfId="38" priority="79" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="79" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J37 I59 F150:F151">
-    <cfRule type="cellIs" dxfId="37" priority="21" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="21" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17015,7 +17009,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA0ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxADoAIABXAGEAcwB0AGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AbABpAGQAIABXAGEAcwB0AGUAIABUAHIAZQBhAHQAbQBlAG4AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXABuAEUAXwBnAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAGcAPQBcAFwAcwB1AG0AXwB0AFwAXABzAHUAbQBfAHcAKABRAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB3AHQAZwApAFwAbgBRAF8AdwB0ACAAPQAgAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAIAAoAHQAKQBcAG4ARQBGAF8AdwB0AGcAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAdAAgAEMATwAyAGUALwB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AdwB0ACwAIABFAEYAXwB3AHQAZwAsAFwAbgAgACAAIAAgAFEAXwB3AHQAIAAqACAARQBGAF8AdwB0AGcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdABcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHcAKABRAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewB3AHQAZwB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzAFwAIgAsACAAXAAiAHQAXAAiACwAIABcACIAUwB1AG0AIABvAGYAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAHcAdABnAFwAIgAsACAAXAAiAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAdAAgAEMATwAyAGUALwB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGcAXAAiACwAIABcACIAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHYAbwBsAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAdgBvAGwAdQBtAGUAIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAdABvAG4AbgBlAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAxADAALgAxAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAG0AYQBzAHMAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AYQBzAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAIAB2AGEAcgBpAGEAYgBsAGUAcwAgAHQAbwAgAGMAbABlAGEAcgBsAHkAIAB0AHIAYQBjAGsAIABpAG4AcAB1AHQAIABvAHIAIABjAGEAbABjAHUAbABhAHQAZQBkACAAUQAgAHYAYQBsAHUAZQBzAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXABuAFEAXwB3AHQAXABuAHQAXABuAFEAXwB3AHQAPQBWAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXABuAFYAXwB3AHQAIAA9ACAAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAG0AMwApAFwAbgBWAFQATQBfAHcAIAA9ACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgACgAdAAvAG0AMwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAXwB3AHQALAAgAFYAVABNAF8AdwAsAFwAbgAgACAAIAAgAFYAXwB3AHQAIAAqACAAVgBUAE0AXwB3AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AdwB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB7AHcAdAB9AD0AVgBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBfAHcAdABcACIALAAgAFwAIgB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgBtADMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFQATQBfAHcAXAAiACwAIABcACIAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgB0AC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBGAHcAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAgAEMATwAyAGUAIAAvACAAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADEAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzADUALAAgADQALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIAB0AHkAcABlACAAdABcACIALAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBFAEYAdwB0AFwAIgAsACAAXAAiAEUARgAgAHMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAyAC4AMQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4ANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAyAC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA0ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUALAAgAGcAcgBlAGUAbgAgAHcAYQBzAHQAZQAsACAAdwBvAG8AZAAsACAAcwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMQA2ADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMwA2ADYANwAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADQAOQAxADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgAxADEAMAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA1ADMANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgA0ADkALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABcAHUAMAAwADIANwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZABcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AHAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAB1ADAAMAAyADcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAFwAdQAwADAAMgA3AHAAcgB1AG4AbgBpAG4AZwBzAFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcAcAByAHUAbgBpAG4AZwBzAFwAdQAwADAAMgA3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAEUARgAgAHMAbwB1AHIAYwBlACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBwAGUAYwBpAGYAaQBjACAAcgBlAGYAZQByAGUAbgBjAGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgAFwAdQAwADAAMgA3AEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuADoAIABGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAdQAwADAAMgA3ACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgAFwAdQAwADAAMgA3AEMAbwBtAHAAbwBzAHQAaQBuAGcAOgAgAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcAHUAMAAwADIANwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAB1ADAAMAAyADcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AVABhAGIAbABlACAAQQAuADQALgAxAC4AMgA6ACAAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzACAAKAB0AC8AbQAzACkAIAAoAFYAVABNAHcAKQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAFQATQB3AFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQALwBtADMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMgAsACAAMgAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBWAFQATQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgA1ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMgA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBvAG8AZABcACIALAAgADAALgAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4ANwAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgB1AGIAYgBlAHIAIABhAG4AZAAgAGwAZQBhAHQAaABlAHIAXAAiACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwAC4ANAAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA2ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbgBzAHQAcgB1AGMAdABpAG8AbgAgAGEAbgBkACAAZABlAG0AbwBsAGkAdABpAG8AbgAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADkAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABDAGgAYQBuAGcAZQBkACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgAgAEMARgB3ACAAdABvACAAVgBUAE0AdwAgAHQAbwAgAG0AYQB0AGMAaAAgAHQAaQB0AGwAZQAgAHYAYQByAGkAYQBiAGwAZQAuAFwAIgApACkAOwBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABUAHkAcABlACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFUAbgBpAHQAVAB5AHAAZQAsAFwAbgAgACAAUwBVAE0ASQBGAFMAKABcAG4AIAAgACAAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgACAAVAByAGUAYQB0AG0AZQBuAHQAQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABUAHkAcABlACwAXABuACAAIAAgACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVwBhAHMAdABlAFQAeQBwAGUALABcAG4AIAAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAXABuACAAIAAgACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAFUAbgBpAHQAVAB5AHAAZQBcAG4AIAAgACkAXABuACkAOwAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17028,14 +17029,7 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA0ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxADoAIABXAGEAcwB0AGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AbABpAGQAIABXAGEAcwB0AGUAIABUAHIAZQBhAHQAbQBlAG4AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXABuAEUAXwBnAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAGcAPQBcAFwAcwB1AG0AXwB0AFwAXABzAHUAbQBfAHcAKABRAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB3AHQAZwApAFwAbgBRAF8AdwB0ACAAPQAgAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAIAAoAHQAKQBcAG4ARQBGAF8AdwB0AGcAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAdAAgAEMATwAyAGUALwB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AdwB0ACwAIABFAEYAXwB3AHQAZwAsAFwAbgAgACAAIAAgAFEAXwB3AHQAIAAqACAARQBGAF8AdwB0AGcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdABcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHcAKABRAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewB3AHQAZwB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzAFwAIgAsACAAXAAiAHQAXAAiACwAIABcACIAUwB1AG0AIABvAGYAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAHcAdABnAFwAIgAsACAAXAAiAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAdAAgAEMATwAyAGUALwB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGcAXAAiACwAIABcACIAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHYAbwBsAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAdgBvAGwAdQBtAGUAIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAdABvAG4AbgBlAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAxADAALgAxAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAG0AYQBzAHMAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AYQBzAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAIAB2AGEAcgBpAGEAYgBsAGUAcwAgAHQAbwAgAGMAbABlAGEAcgBsAHkAIAB0AHIAYQBjAGsAIABpAG4AcAB1AHQAIABvAHIAIABjAGEAbABjAHUAbABhAHQAZQBkACAAUQAgAHYAYQBsAHUAZQBzAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXABuAFEAXwB3AHQAXABuAHQAXABuAFEAXwB3AHQAPQBWAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXABuAFYAXwB3AHQAIAA9ACAAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAG0AMwApAFwAbgBWAFQATQBfAHcAIAA9ACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgACgAdAAvAG0AMwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAXwB3AHQALAAgAFYAVABNAF8AdwAsAFwAbgAgACAAIAAgAFYAXwB3AHQAIAAqACAAVgBUAE0AXwB3AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AdwB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB7AHcAdAB9AD0AVgBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBfAHcAdABcACIALAAgAFwAIgB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgBtADMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFQATQBfAHcAXAAiACwAIABcACIAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgB0AC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBGAHcAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAgAEMATwAyAGUAIAAvACAAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADEAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzADUALAAgADQALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIAB0AHkAcABlACAAdABcACIALAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBFAEYAdwB0AFwAIgAsACAAXAAiAEUARgAgAHMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAyAC4AMQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4ANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAyAC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA0ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUALAAgAGcAcgBlAGUAbgAgAHcAYQBzAHQAZQAsACAAdwBvAG8AZAAsACAAcwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMQA2ADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMwA2ADYANwAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADQAOQAxADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgAxADEAMAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA1ADMANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgA0ADkALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgAwADQANgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgAwADIAOAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABcAHUAMAAwADIANwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZABcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AHAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAB1ADAAMAAyADcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAFwAdQAwADAAMgA3AHAAcgB1AG4AbgBpAG4AZwBzAFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcAcAByAHUAbgBpAG4AZwBzAFwAdQAwADAAMgA3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAEUARgAgAHMAbwB1AHIAYwBlACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBwAGUAYwBpAGYAaQBjACAAcgBlAGYAZQByAGUAbgBjAGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgAFwAdQAwADAAMgA3AEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuADoAIABGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAdQAwADAAMgA3ACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABzAHUAYgAtAGMAYQB0AGUAZwBvAHIAaQBlAHMAIABmAG8AcgAgAFwAdQAwADAAMgA3AEMAbwBtAHAAbwBzAHQAaQBuAGcAOgAgAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcAHUAMAAwADIANwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAB1ADAAMAAyADcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AVABhAGIAbABlACAAQQAuADQALgAxAC4AMgA6ACAAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzACAAKAB0AC8AbQAzACkAIAAoAFYAVABNAHcAKQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAFQATQB3AFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQALwBtADMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMgAsACAAMgAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBWAFQATQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADAALgA1ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIAAwAC4AMgA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBvAG8AZABcACIALAAgADAALgAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIAAwAC4ANwAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgB1AGIAYgBlAHIAIABhAG4AZAAgAGwAZQBhAHQAaABlAHIAXAAiACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwAC4ANAAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA2ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbgBzAHQAcgB1AGMAdABpAG8AbgAgAGEAbgBkACAAZABlAG0AbwBsAGkAdABpAG8AbgAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADkAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABDAGgAYQBuAGcAZQBkACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgAgAEMARgB3ACAAdABvACAAVgBUAE0AdwAgAHQAbwAgAG0AYQB0AGMAaAAgAHQAaQB0AGwAZQAgAHYAYQByAGkAYQBiAGwAZQAuAFwAIgApACkAOwBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABUAHkAcABlACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFUAbgBpAHQAVAB5AHAAZQAsAFwAbgAgACAAUwBVAE0ASQBGAFMAKABcAG4AIAAgACAAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgACAAVAByAGUAYQB0AG0AZQBuAHQAQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABUAHkAcABlACwAXABuACAAIAAgACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVwBhAHMAdABlAFQAeQBwAGUALABcAG4AIAAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAXABuACAAIAAgACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAFUAbgBpAHQAVAB5AHAAZQBcAG4AIAAgACkAXABuACkAOwAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17234,9 +17228,12 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17250,12 +17247,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>